<commit_message>
Radar: większy, pierścień na podtyp (dealer/salon/serwis), ikona klienta, etykieta bez nakładania; podtypy w danych i filtrach A/B/C
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/macierz-demo.xlsx
+++ b/macierz-demo.xlsx
@@ -12,7 +12,7 @@
     <sheet name="akcje" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'punkty_styku'!$A$1:$K$61</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'punkty_styku'!$A$1:$L$61</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'cechy'!$A$1:$E$360</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'akcje'!$A$1:$J$56</definedName>
   </definedNames>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K61"/>
+  <dimension ref="A1:L61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -446,6 +446,7 @@
     <col width="27" customWidth="1" min="9" max="9"/>
     <col width="17" customWidth="1" min="10" max="10"/>
     <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -504,6 +505,11 @@
           <t>status_danych</t>
         </is>
       </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>podtyp</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -561,6 +567,7 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -618,6 +625,7 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -675,6 +683,7 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -732,6 +741,7 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -789,6 +799,7 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -846,6 +857,7 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -903,6 +915,7 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -960,6 +973,7 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1017,6 +1031,7 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1062,6 +1077,7 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1119,6 +1135,7 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1176,6 +1193,7 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1233,6 +1251,7 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1290,6 +1309,7 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1347,6 +1367,7 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1404,6 +1425,7 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1461,6 +1483,7 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1518,6 +1541,7 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1575,6 +1599,7 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1632,6 +1657,7 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1689,6 +1715,7 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1746,6 +1773,7 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1803,6 +1831,7 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1860,6 +1889,7 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1917,6 +1947,7 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1974,6 +2005,7 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2031,6 +2063,7 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2088,6 +2121,7 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2145,6 +2179,7 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2202,6 +2237,7 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2259,6 +2295,11 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>dealer</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2316,6 +2357,11 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>salon</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2373,6 +2419,11 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>salon</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2430,6 +2481,11 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L35" s="2" t="inlineStr">
+        <is>
+          <t>salon</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2487,6 +2543,11 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>salon</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2544,6 +2605,11 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L37" s="2" t="inlineStr">
+        <is>
+          <t>salon</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2601,6 +2667,11 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>salon</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -2658,6 +2729,11 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L39" s="2" t="inlineStr">
+        <is>
+          <t>salon</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -2715,6 +2791,11 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L40" s="2" t="inlineStr">
+        <is>
+          <t>salon</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -2772,6 +2853,11 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L41" s="2" t="inlineStr">
+        <is>
+          <t>salon</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -2829,6 +2915,11 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L42" s="2" t="inlineStr">
+        <is>
+          <t>dealer</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -2886,6 +2977,11 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L43" s="2" t="inlineStr">
+        <is>
+          <t>dealer</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -2943,6 +3039,11 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L44" s="2" t="inlineStr">
+        <is>
+          <t>salon</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -3000,6 +3101,11 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L45" s="2" t="inlineStr">
+        <is>
+          <t>salon</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -3057,6 +3163,11 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L46" s="2" t="inlineStr">
+        <is>
+          <t>salon</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -3114,6 +3225,11 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L47" s="2" t="inlineStr">
+        <is>
+          <t>dealer</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -3171,6 +3287,11 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L48" s="2" t="inlineStr">
+        <is>
+          <t>serwis</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -3228,6 +3349,11 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L49" s="2" t="inlineStr">
+        <is>
+          <t>serwis</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -3285,6 +3411,11 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L50" s="2" t="inlineStr">
+        <is>
+          <t>serwis</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -3342,6 +3473,11 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L51" s="2" t="inlineStr">
+        <is>
+          <t>serwis</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -3399,6 +3535,11 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L52" s="2" t="inlineStr">
+        <is>
+          <t>serwis</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -3456,6 +3597,11 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L53" s="2" t="inlineStr">
+        <is>
+          <t>serwis</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -3511,6 +3657,11 @@
       <c r="K54" s="2" t="inlineStr">
         <is>
           <t>DEMO</t>
+        </is>
+      </c>
+      <c r="L54" s="2" t="inlineStr">
+        <is>
+          <t>serwis</t>
         </is>
       </c>
     </row>
@@ -3558,6 +3709,11 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L55" s="2" t="inlineStr">
+        <is>
+          <t>serwis</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -3615,6 +3771,11 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L56" s="2" t="inlineStr">
+        <is>
+          <t>serwis</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -3672,6 +3833,11 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L57" s="2" t="inlineStr">
+        <is>
+          <t>serwis</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -3729,6 +3895,11 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L58" s="2" t="inlineStr">
+        <is>
+          <t>serwis</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -3786,6 +3957,11 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L59" s="2" t="inlineStr">
+        <is>
+          <t>serwis</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -3843,6 +4019,11 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L60" s="2" t="inlineStr">
+        <is>
+          <t>dealer</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -3900,9 +4081,14 @@
           <t>DEMO</t>
         </is>
       </c>
+      <c r="L61" s="2" t="inlineStr">
+        <is>
+          <t>dealer</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K61"/>
+  <autoFilter ref="A1:L61"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Macierz: paski na kafelku pokazują stopień zaopiekowania 1-5 (kolor oceny) zamiast emocji; pole care w danych DEMO
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/macierz-demo.xlsx
+++ b/macierz-demo.xlsx
@@ -12,7 +12,7 @@
     <sheet name="akcje" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'punkty_styku'!$A$1:$L$61</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'punkty_styku'!$A$1:$M$61</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'cechy'!$A$1:$E$360</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'akcje'!$A$1:$J$56</definedName>
   </definedNames>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L61"/>
+  <dimension ref="A1:M61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -447,6 +447,7 @@
     <col width="17" customWidth="1" min="10" max="10"/>
     <col width="15" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="19" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -510,6 +511,11 @@
           <t>podtyp</t>
         </is>
       </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>zaopiekowanie_1_5</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -568,6 +574,9 @@
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -626,6 +635,9 @@
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr"/>
+      <c r="M3" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -684,6 +696,9 @@
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -742,6 +757,9 @@
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr"/>
+      <c r="M5" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -800,6 +818,9 @@
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr"/>
+      <c r="M6" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -858,6 +879,9 @@
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr"/>
+      <c r="M7" s="2" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -916,6 +940,9 @@
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr"/>
+      <c r="M8" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -974,6 +1001,9 @@
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr"/>
+      <c r="M9" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1032,6 +1062,9 @@
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr"/>
+      <c r="M10" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1078,6 +1111,7 @@
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr"/>
+      <c r="M11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1136,6 +1170,9 @@
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr"/>
+      <c r="M12" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1194,6 +1231,9 @@
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr"/>
+      <c r="M13" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1252,6 +1292,9 @@
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr"/>
+      <c r="M14" s="2" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1310,6 +1353,9 @@
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr"/>
+      <c r="M15" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1368,6 +1414,9 @@
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr"/>
+      <c r="M16" s="2" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1426,6 +1475,9 @@
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr"/>
+      <c r="M17" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1484,6 +1536,9 @@
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr"/>
+      <c r="M18" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1542,6 +1597,9 @@
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr"/>
+      <c r="M19" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1600,6 +1658,9 @@
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr"/>
+      <c r="M20" s="2" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1658,6 +1719,9 @@
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr"/>
+      <c r="M21" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1716,6 +1780,9 @@
         </is>
       </c>
       <c r="L22" s="2" t="inlineStr"/>
+      <c r="M22" s="2" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1774,6 +1841,9 @@
         </is>
       </c>
       <c r="L23" s="2" t="inlineStr"/>
+      <c r="M23" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1832,6 +1902,9 @@
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr"/>
+      <c r="M24" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1890,6 +1963,9 @@
         </is>
       </c>
       <c r="L25" s="2" t="inlineStr"/>
+      <c r="M25" s="2" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1948,6 +2024,9 @@
         </is>
       </c>
       <c r="L26" s="2" t="inlineStr"/>
+      <c r="M26" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2006,6 +2085,9 @@
         </is>
       </c>
       <c r="L27" s="2" t="inlineStr"/>
+      <c r="M27" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2064,6 +2146,9 @@
         </is>
       </c>
       <c r="L28" s="2" t="inlineStr"/>
+      <c r="M28" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2122,6 +2207,9 @@
         </is>
       </c>
       <c r="L29" s="2" t="inlineStr"/>
+      <c r="M29" s="2" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2180,6 +2268,9 @@
         </is>
       </c>
       <c r="L30" s="2" t="inlineStr"/>
+      <c r="M30" s="2" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2238,6 +2329,9 @@
         </is>
       </c>
       <c r="L31" s="2" t="inlineStr"/>
+      <c r="M31" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2300,6 +2394,9 @@
           <t>dealer</t>
         </is>
       </c>
+      <c r="M32" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2362,6 +2459,9 @@
           <t>salon</t>
         </is>
       </c>
+      <c r="M33" s="2" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2424,6 +2524,9 @@
           <t>salon</t>
         </is>
       </c>
+      <c r="M34" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2486,6 +2589,9 @@
           <t>salon</t>
         </is>
       </c>
+      <c r="M35" s="2" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2548,6 +2654,9 @@
           <t>salon</t>
         </is>
       </c>
+      <c r="M36" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2610,6 +2719,9 @@
           <t>salon</t>
         </is>
       </c>
+      <c r="M37" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2672,6 +2784,9 @@
           <t>salon</t>
         </is>
       </c>
+      <c r="M38" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -2734,6 +2849,9 @@
           <t>salon</t>
         </is>
       </c>
+      <c r="M39" s="2" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -2796,6 +2914,9 @@
           <t>salon</t>
         </is>
       </c>
+      <c r="M40" s="2" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -2858,6 +2979,9 @@
           <t>salon</t>
         </is>
       </c>
+      <c r="M41" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -2920,6 +3044,9 @@
           <t>dealer</t>
         </is>
       </c>
+      <c r="M42" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -2982,6 +3109,9 @@
           <t>dealer</t>
         </is>
       </c>
+      <c r="M43" s="2" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -3044,6 +3174,9 @@
           <t>salon</t>
         </is>
       </c>
+      <c r="M44" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -3106,6 +3239,9 @@
           <t>salon</t>
         </is>
       </c>
+      <c r="M45" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -3168,6 +3304,9 @@
           <t>salon</t>
         </is>
       </c>
+      <c r="M46" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -3230,6 +3369,9 @@
           <t>dealer</t>
         </is>
       </c>
+      <c r="M47" s="2" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -3292,6 +3434,9 @@
           <t>serwis</t>
         </is>
       </c>
+      <c r="M48" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -3354,6 +3499,9 @@
           <t>serwis</t>
         </is>
       </c>
+      <c r="M49" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -3416,6 +3564,9 @@
           <t>serwis</t>
         </is>
       </c>
+      <c r="M50" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -3478,6 +3629,9 @@
           <t>serwis</t>
         </is>
       </c>
+      <c r="M51" s="2" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -3540,6 +3694,9 @@
           <t>serwis</t>
         </is>
       </c>
+      <c r="M52" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -3602,6 +3759,9 @@
           <t>serwis</t>
         </is>
       </c>
+      <c r="M53" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -3663,6 +3823,9 @@
         <is>
           <t>serwis</t>
         </is>
+      </c>
+      <c r="M54" s="2" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="55">
@@ -3714,6 +3877,7 @@
           <t>serwis</t>
         </is>
       </c>
+      <c r="M55" s="2" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -3776,6 +3940,9 @@
           <t>serwis</t>
         </is>
       </c>
+      <c r="M56" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -3838,6 +4005,9 @@
           <t>serwis</t>
         </is>
       </c>
+      <c r="M57" s="2" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -3900,6 +4070,9 @@
           <t>serwis</t>
         </is>
       </c>
+      <c r="M58" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -3962,6 +4135,9 @@
           <t>serwis</t>
         </is>
       </c>
+      <c r="M59" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -4024,6 +4200,9 @@
           <t>dealer</t>
         </is>
       </c>
+      <c r="M60" s="2" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -4086,9 +4265,12 @@
           <t>dealer</t>
         </is>
       </c>
+      <c r="M61" s="2" t="n">
+        <v>2</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L61"/>
+  <autoFilter ref="A1:M61"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Dane: macierz-demo.xlsx źródłem danych; konwerter xlsx->CSV+data/matrix.js (stdlib), walidacja z arkuszem i wierszem, test; generator jako jednorazowy seed
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/macierz-demo.xlsx
+++ b/macierz-demo.xlsx
@@ -10,11 +10,15 @@
     <sheet name="punkty_styku" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="cechy" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="akcje" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="slowniki" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="procesy" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'punkty_styku'!$A$1:$M$61</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'cechy'!$A$1:$E$360</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'akcje'!$A$1:$J$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'slowniki'!$A$1:$C$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'procesy'!$A$1:$B$15</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -16844,4 +16848,535 @@
   <autoFilter ref="A1:J56"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>grupa</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>klucz</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>etykieta</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>matrix</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>importer</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Importer</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>matrix</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>dealer</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Dealer i serwis</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>subtype</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>dealer</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Dealer</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>subtype</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>salon</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Salon</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>subtype</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>serwis</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Serwis</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>rating</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>niezaopiekowany</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Niezaopiekowany</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>rating</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>do_poprawy</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Do poprawy</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>rating</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>W porządku</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>rating</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>brak_oceny</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Brak oceny</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>monitoring</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Monitorowany</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>monitoring</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>częściowo</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Monitorowany częściowo</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>monitoring</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>nie</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Niemonitorowany</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>featureType</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>dobra_praktyka</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Dobre praktyki</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>featureType</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>blad_typowy</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Błędy typowe</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>featureType</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>blad_diagnozowany</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Błędy diagnozowane</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>featureType</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>przyklad</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Przykłady z życia</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>featureType</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>zrodlo</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Źródła danych</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>actionKind</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>quick_win</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Quick win</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>actionKind</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>docelowa</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Usprawnienie docelowe</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:C20"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>lp</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>nazwa</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Pozyskanie</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Zapytanie</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Zakup</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Finansowanie</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Zamówienie</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Dostawa</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Użytkowanie</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Serwis</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Posprzedaż</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Gwarancja</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Reklamacje</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Auta używane</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Lojalność</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Wymiana</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B15"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Mapa przepływu (dane): zakładki nastepne/przypadki/kroki_przypadku, tory z danych, flow-core (walidacja), dane DEMO, dwuklik konwertera
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/macierz-demo.xlsx
+++ b/macierz-demo.xlsx
@@ -12,13 +12,19 @@
     <sheet name="akcje" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="slowniki" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="procesy" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="nastepne" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="przypadki" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="kroki_przypadku" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'punkty_styku'!$A$1:$M$61</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'punkty_styku'!$A$1:$N$61</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'cechy'!$A$1:$E$360</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'akcje'!$A$1:$J$56</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'slowniki'!$A$1:$C$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'slowniki'!$A$1:$C$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'procesy'!$A$1:$B$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'nastepne'!$A$1:$E$84</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'przypadki'!$A$1:$F$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'kroki_przypadku'!$A$1:$F$31</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -436,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M61"/>
+  <dimension ref="A1:N61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -452,6 +458,7 @@
     <col width="15" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
     <col width="19" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -520,6 +527,11 @@
           <t>zaopiekowanie_1_5</t>
         </is>
       </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>tor_nadpisanie</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -581,6 +593,7 @@
       <c r="M2" s="2" t="n">
         <v>4</v>
       </c>
+      <c r="N2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -642,6 +655,7 @@
       <c r="M3" s="2" t="n">
         <v>3</v>
       </c>
+      <c r="N3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -703,6 +717,7 @@
       <c r="M4" s="2" t="n">
         <v>1</v>
       </c>
+      <c r="N4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -764,6 +779,7 @@
       <c r="M5" s="2" t="n">
         <v>3</v>
       </c>
+      <c r="N5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -825,6 +841,7 @@
       <c r="M6" s="2" t="n">
         <v>3</v>
       </c>
+      <c r="N6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -886,6 +903,7 @@
       <c r="M7" s="2" t="n">
         <v>2</v>
       </c>
+      <c r="N7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -947,6 +965,7 @@
       <c r="M8" s="2" t="n">
         <v>3</v>
       </c>
+      <c r="N8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1008,6 +1027,7 @@
       <c r="M9" s="2" t="n">
         <v>3</v>
       </c>
+      <c r="N9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1069,6 +1089,7 @@
       <c r="M10" s="2" t="n">
         <v>3</v>
       </c>
+      <c r="N10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1116,6 +1137,7 @@
       </c>
       <c r="L11" s="2" t="inlineStr"/>
       <c r="M11" s="2" t="inlineStr"/>
+      <c r="N11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1177,6 +1199,7 @@
       <c r="M12" s="2" t="n">
         <v>3</v>
       </c>
+      <c r="N12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1238,6 +1261,7 @@
       <c r="M13" s="2" t="n">
         <v>5</v>
       </c>
+      <c r="N13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1299,6 +1323,7 @@
       <c r="M14" s="2" t="n">
         <v>1</v>
       </c>
+      <c r="N14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1360,6 +1385,7 @@
       <c r="M15" s="2" t="n">
         <v>3</v>
       </c>
+      <c r="N15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1421,6 +1447,7 @@
       <c r="M16" s="2" t="n">
         <v>2</v>
       </c>
+      <c r="N16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1482,6 +1509,7 @@
       <c r="M17" s="2" t="n">
         <v>4</v>
       </c>
+      <c r="N17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1543,6 +1571,7 @@
       <c r="M18" s="2" t="n">
         <v>3</v>
       </c>
+      <c r="N18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1604,6 +1633,7 @@
       <c r="M19" s="2" t="n">
         <v>3</v>
       </c>
+      <c r="N19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1665,6 +1695,7 @@
       <c r="M20" s="2" t="n">
         <v>1</v>
       </c>
+      <c r="N20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1726,6 +1757,7 @@
       <c r="M21" s="2" t="n">
         <v>5</v>
       </c>
+      <c r="N21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1787,6 +1819,7 @@
       <c r="M22" s="2" t="n">
         <v>2</v>
       </c>
+      <c r="N22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1848,6 +1881,7 @@
       <c r="M23" s="2" t="n">
         <v>4</v>
       </c>
+      <c r="N23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1909,6 +1943,7 @@
       <c r="M24" s="2" t="n">
         <v>3</v>
       </c>
+      <c r="N24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1970,6 +2005,7 @@
       <c r="M25" s="2" t="n">
         <v>1</v>
       </c>
+      <c r="N25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2031,6 +2067,7 @@
       <c r="M26" s="2" t="n">
         <v>5</v>
       </c>
+      <c r="N26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2092,6 +2129,7 @@
       <c r="M27" s="2" t="n">
         <v>3</v>
       </c>
+      <c r="N27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2153,6 +2191,7 @@
       <c r="M28" s="2" t="n">
         <v>4</v>
       </c>
+      <c r="N28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2214,6 +2253,7 @@
       <c r="M29" s="2" t="n">
         <v>2</v>
       </c>
+      <c r="N29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2275,6 +2315,7 @@
       <c r="M30" s="2" t="n">
         <v>1</v>
       </c>
+      <c r="N30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2336,6 +2377,7 @@
       <c r="M31" s="2" t="n">
         <v>3</v>
       </c>
+      <c r="N31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2401,6 +2443,7 @@
       <c r="M32" s="2" t="n">
         <v>3</v>
       </c>
+      <c r="N32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2466,6 +2509,7 @@
       <c r="M33" s="2" t="n">
         <v>2</v>
       </c>
+      <c r="N33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2531,6 +2575,7 @@
       <c r="M34" s="2" t="n">
         <v>5</v>
       </c>
+      <c r="N34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2596,6 +2641,7 @@
       <c r="M35" s="2" t="n">
         <v>1</v>
       </c>
+      <c r="N35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2661,6 +2707,7 @@
       <c r="M36" s="2" t="n">
         <v>4</v>
       </c>
+      <c r="N36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2726,6 +2773,7 @@
       <c r="M37" s="2" t="n">
         <v>5</v>
       </c>
+      <c r="N37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2791,6 +2839,7 @@
       <c r="M38" s="2" t="n">
         <v>4</v>
       </c>
+      <c r="N38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -2856,6 +2905,7 @@
       <c r="M39" s="2" t="n">
         <v>2</v>
       </c>
+      <c r="N39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -2921,6 +2971,7 @@
       <c r="M40" s="2" t="n">
         <v>1</v>
       </c>
+      <c r="N40" s="2" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -2986,6 +3037,7 @@
       <c r="M41" s="2" t="n">
         <v>3</v>
       </c>
+      <c r="N41" s="2" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -3051,6 +3103,7 @@
       <c r="M42" s="2" t="n">
         <v>3</v>
       </c>
+      <c r="N42" s="2" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -3116,6 +3169,7 @@
       <c r="M43" s="2" t="n">
         <v>2</v>
       </c>
+      <c r="N43" s="2" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -3181,6 +3235,7 @@
       <c r="M44" s="2" t="n">
         <v>5</v>
       </c>
+      <c r="N44" s="2" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -3246,6 +3301,7 @@
       <c r="M45" s="2" t="n">
         <v>4</v>
       </c>
+      <c r="N45" s="2" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -3311,6 +3367,7 @@
       <c r="M46" s="2" t="n">
         <v>3</v>
       </c>
+      <c r="N46" s="2" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -3376,6 +3433,7 @@
       <c r="M47" s="2" t="n">
         <v>1</v>
       </c>
+      <c r="N47" s="2" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -3441,6 +3499,7 @@
       <c r="M48" s="2" t="n">
         <v>3</v>
       </c>
+      <c r="N48" s="2" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -3506,6 +3565,7 @@
       <c r="M49" s="2" t="n">
         <v>3</v>
       </c>
+      <c r="N49" s="2" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -3571,6 +3631,7 @@
       <c r="M50" s="2" t="n">
         <v>3</v>
       </c>
+      <c r="N50" s="2" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -3636,6 +3697,7 @@
       <c r="M51" s="2" t="n">
         <v>2</v>
       </c>
+      <c r="N51" s="2" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -3701,6 +3763,7 @@
       <c r="M52" s="2" t="n">
         <v>5</v>
       </c>
+      <c r="N52" s="2" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -3766,6 +3829,7 @@
       <c r="M53" s="2" t="n">
         <v>3</v>
       </c>
+      <c r="N53" s="2" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -3831,6 +3895,7 @@
       <c r="M54" s="2" t="n">
         <v>1</v>
       </c>
+      <c r="N54" s="2" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -3882,6 +3947,7 @@
         </is>
       </c>
       <c r="M55" s="2" t="inlineStr"/>
+      <c r="N55" s="2" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -3947,6 +4013,7 @@
       <c r="M56" s="2" t="n">
         <v>4</v>
       </c>
+      <c r="N56" s="2" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -4012,6 +4079,7 @@
       <c r="M57" s="2" t="n">
         <v>2</v>
       </c>
+      <c r="N57" s="2" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -4077,6 +4145,7 @@
       <c r="M58" s="2" t="n">
         <v>3</v>
       </c>
+      <c r="N58" s="2" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -4142,6 +4211,7 @@
       <c r="M59" s="2" t="n">
         <v>3</v>
       </c>
+      <c r="N59" s="2" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -4207,6 +4277,7 @@
       <c r="M60" s="2" t="n">
         <v>1</v>
       </c>
+      <c r="N60" s="2" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -4272,9 +4343,10 @@
       <c r="M61" s="2" t="n">
         <v>2</v>
       </c>
+      <c r="N61" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M61"/>
+  <autoFilter ref="A1:N61"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -16856,7 +16928,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -17204,8 +17276,76 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>stan</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>zadzialal</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Zadziałał</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>stan</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>czesciowo</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Częściowo</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>stan</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>nie_zadzialal</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Nie zadziałał</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>stan</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>brakuje</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Brakuje</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C20"/>
+  <autoFilter ref="A1:C24"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -17379,4 +17519,3120 @@
   <autoFilter ref="A1:B15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E84"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>punkt_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>nastepny_id</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>etykieta</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>opcjonalny</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>status_danych</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>imp-01</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>imp-04</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr"/>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>nie</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>imp-02</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>imp-04</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr"/>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>nie</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>imp-03</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>dea-01</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>kontakty z targów</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>nie</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>imp-04</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>imp-05</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr"/>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>nie</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>imp-04</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>imp-06</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr"/>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>imp-04</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>imp-07</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>pytanie o ofertę</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>imp-04</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>imp-08</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>czat</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>imp-04</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>imp-09</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>finansowanie</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>imp-05</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>dea-01</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>zapytanie</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>nie</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>imp-05</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>dea-07</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>umów jazdę</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>imp-06</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>dea-02</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr"/>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>nie</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>imp-07</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>dea-01</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr"/>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>nie</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>imp-08</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>dea-03</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr"/>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>nie</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>imp-09</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>dea-11</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr"/>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>dea-01</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>dea-04</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr"/>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>nie</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>dea-02</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>dea-04</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr"/>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>nie</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>dea-03</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>dea-04</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr"/>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>nie</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>dea-04</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>dea-05</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr"/>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>nie</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>dea-05</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>dea-06</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr"/>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>nie</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>dea-06</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>dea-07</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr"/>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>dea-06</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>dea-08</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr"/>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>nie</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>dea-07</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>dea-08</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr"/>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>nie</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>dea-08</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>dea-09</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr"/>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>dea-08</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>dea-10</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr"/>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>dea-08</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>dea-11</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr"/>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>dea-08</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>dea-12</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr"/>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>nie</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>dea-09</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>dea-12</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr"/>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>nie</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>dea-10</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>dea-12</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr"/>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>nie</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>dea-11</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>dea-12</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr"/>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>nie</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>dea-11</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>imp-10</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>ubezpieczenie</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>dea-11</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>imp-11</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>wniosek</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>imp-10</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>dea-12</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr"/>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>nie</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>imp-11</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>dea-12</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr"/>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>nie</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>dea-12</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>imp-12</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr"/>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>nie</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>imp-12</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>imp-13</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr"/>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>nie</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>imp-13</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>imp-14</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>gdy opóźnienie</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>imp-13</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>dea-13</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr"/>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>nie</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>imp-14</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>dea-13</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr"/>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>nie</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>dea-13</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>dea-14</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr"/>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>nie</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>dea-14</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>imp-15</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr"/>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>dea-14</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>imp-16</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr"/>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>dea-14</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>dea-15</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr"/>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>nie</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>dea-15</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>dea-16</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr"/>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>nie</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>imp-15</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>imp-17</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr"/>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>nie</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>imp-16</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>imp-17</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr"/>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>nie</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>dea-16</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>imp-17</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr"/>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>nie</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>dea-16</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>imp-25</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr"/>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>imp-17</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>imp-18</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr"/>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>imp-17</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>imp-19</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr"/>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>imp-17</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>imp-20</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>awaria</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>imp-17</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>imp-21</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr"/>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>imp-17</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>imp-22</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr"/>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>imp-17</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>imp-24</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>wada</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>imp-21</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>dea-17</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr"/>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>imp-22</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>dea-17</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr"/>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>nie</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>imp-17</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>dea-17</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr"/>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>nie</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>dea-17</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>dea-18</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr"/>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>nie</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>dea-17</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>dea-28</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>po wypadku</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>dea-18</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>dea-19</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr"/>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>nie</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>dea-18</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>dea-21</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr"/>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>dea-18</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>dea-22</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr"/>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>dea-18</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>dea-27</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>gwarancja</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>dea-19</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>dea-20</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr"/>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>dea-19</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>dea-23</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr"/>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>nie</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>dea-20</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>dea-23</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr"/>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>nie</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>dea-21</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>dea-23</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr"/>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>nie</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>dea-22</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>dea-23</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr"/>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>nie</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>dea-28</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>dea-19</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr"/>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>nie</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>dea-23</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>dea-24</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr"/>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>nie</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>dea-24</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>dea-25</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr"/>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>nie</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>dea-25</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>dea-26</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr"/>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>nie</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>dea-26</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>imp-22</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>kolejny przegląd</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>dea-26</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>imp-26</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr"/>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>dea-27</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>imp-23</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>odwołanie</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>imp-23</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>imp-24</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr"/>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>imp-25</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>imp-26</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr"/>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>nie</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>imp-26</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>imp-27</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr"/>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>imp-26</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>imp-28</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr"/>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>imp-26</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>dea-30</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr"/>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>dea-30</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>imp-30</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr"/>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>nie</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>imp-30</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>imp-29</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr"/>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>nie</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>imp-29</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>dea-29</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr"/>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>imp-29</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>dea-01</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>kolejny zakup</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E84"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="29" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>przypadek_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>nazwa</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>klient</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>model_pojazdu</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>numer_sprawy</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>status_danych</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>P-01</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Zakup z jazdą próbną</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Klient DEMO A</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Model DEMO X</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>DEMO-001</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>P-02</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Serwis z niespodzianką</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Klient DEMO B</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Model DEMO Y</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>DEMO-002</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>P-03</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Odmowa naprawy gwarancyjnej</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr"/>
+      <c r="D4" s="2" t="inlineStr"/>
+      <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F4"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="58" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>przypadek_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>lp</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>punkt_id</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>stan</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>co_sie_stalo</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>status_danych</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>P-01</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>imp-01</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>zadzialal</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Klient słyszy spot i zapamiętuje markę.</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>P-01</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>imp-04</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>zadzialal</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Na stronie znajduje model i orientacyjną cenę.</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>P-01</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>imp-05</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>czesciowo</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Konfiguruje auto, ale nie widzi jak umówić jazdę.</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>P-01</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>dea-01</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>nie_zadzialal</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Wysyła zapytanie, odpowiedź przychodzi po trzech dniach.</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>P-01</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>dea-04</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>zadzialal</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>W salonie zostaje powitany po minucie.</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>P-01</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>dea-05</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>zadzialal</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Doradca pyta o dojazdy i potrzeby rodziny.</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>P-01</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>dea-06</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>zadzialal</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Prezentacja skupia się na tym, co ważne dla klienta.</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>P-01</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>dea-07</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>zadzialal</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Jazda po trasie zbliżonej do codziennych dojazdów.</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>P-01</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>dea-08</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>czesciowo</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Oferta jest czytelna, ale bez wyjaśnienia dodatków.</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>P-01</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>dea-12</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>czesciowo</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Podpisanie trwa dwie godziny, dane trzeba przepisywać.</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>P-01</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>imp-12</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>zadzialal</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Potwierdzenie przychodzi od razu, ale bez terminu.</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>P-01</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>imp-13</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>nie_zadzialal</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Przez kilka miesięcy brak informacji o statusie.</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>P-01</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>imp-14</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>nie_zadzialal</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>O opóźnieniu klient dowiaduje się w dniu dostawy.</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>P-01</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>dea-13</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>zadzialal</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Auto czeka umyte i kompletne.</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>P-01</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>dea-14</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>zadzialal</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Uroczyste wydanie kluczyków.</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>P-01</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>dea-15</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>czesciowo</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Doradca pokazuje tylko kilka funkcji.</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>P-01</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>dea-16</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>brakuje</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Po wydaniu auta nikt się nie odzywa.</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>P-02</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>dea-17</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>czesciowo</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Rezerwacja tylko telefoniczna, trzy próby.</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>P-02</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>dea-18</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>czesciowo</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Przyjęcie bez potwierdzenia kosztu.</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>P-02</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>dea-19</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>zadzialal</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Kosztorys z opisem prac.</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>P-02</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>dea-20</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>nie_zadzialal</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Prace dodatkowe wykonane bez zgody klienta.</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>P-02</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>dea-23</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>brakuje</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Brak informacji o postępie prac.</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>P-02</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>dea-24</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>zadzialal</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Odbiór bez kolejki.</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>P-02</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>dea-25</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>czesciowo</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Faktura wyższa od kosztorysu, pytania o pozycje.</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>P-02</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>dea-26</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>brakuje</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Po odbiorze brak kontaktu z serwisu.</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>P-03</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>dea-17</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>zadzialal</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Rezerwacja online bez problemu.</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>P-03</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>dea-18</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>czesciowo</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Doradca przyjmuje auto, nie omawia zasad gwarancji.</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>P-03</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>dea-27</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>nie_zadzialal</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Odmowa naprawy bez uzasadnienia.</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>P-03</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>imp-23</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>nie_zadzialal</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Importer odsyła sprawę bez decyzji.</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>P-03</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>imp-24</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>nie_zadzialal</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Sprawa wędruje między działami.</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F31"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
xlsx: zakładka czytaj_mnie i listy rozwijane (słowniki, ID punktów, skale); emocja_1_5 jako liczba
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/macierz-demo.xlsx
+++ b/macierz-demo.xlsx
@@ -7,24 +7,25 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="punkty_styku" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="cechy" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="akcje" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="slowniki" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="procesy" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="nastepne" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="przypadki" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="kroki_przypadku" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="czytaj_mnie" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="punkty_styku" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="cechy" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="akcje" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="slowniki" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="procesy" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="nastepne" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="przypadki" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="kroki_przypadku" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'punkty_styku'!$A$1:$N$61</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'cechy'!$A$1:$E$360</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'akcje'!$A$1:$J$56</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'slowniki'!$A$1:$C$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'procesy'!$A$1:$B$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'nastepne'!$A$1:$E$84</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'przypadki'!$A$1:$F$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'kroki_przypadku'!$A$1:$F$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'punkty_styku'!$A$1:$N$61</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'cechy'!$A$1:$E$360</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'akcje'!$A$1:$J$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'slowniki'!$A$1:$C$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'procesy'!$A$1:$B$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'nastepne'!$A$1:$E$84</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'przypadki'!$A$1:$F$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'kroki_przypadku'!$A$1:$F$31</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -33,7 +34,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -44,6 +45,17 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -71,12 +83,21 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -439,6 +460,170 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00041428"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="110" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>CZYTAJ MNIE: jak uzupełniać ten plik</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr"/>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Ten plik jest źródłem danych dla wizualizacji (macierz, priorytety, radar, mapa przepływu). Zielone zakładki wypełniasz Ty, szare (slowniki, procesy) zmieniasz tylko przy nowym torze, stanie albo procesie.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Kolejność pracy</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>punkty_styku: jeden wiersz na punkt styku. Nadaj unikalne ID (np. imp-01). Proces, ocenę, monitoring i macierz wybierz z listy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>cechy i akcje: wiele wierszy na punkt. W kolumnie punkt_id wybierz ID z listy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>nastepne: mapa przepływu. Jeden wiersz = krok z punktu (punkt_id) do kolejnego (nastepny_id). Kilka wierszy z tym samym punkt_id to rozwidlenie. Opcjonalny = tak, jeśli krok można pominąć. Powroty do wcześniejszego punktu są dozwolone.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>przypadki: prawdziwy przebieg klienta (nazwa wymagana; klient, model_pojazdu i numer_sprawy opcjonalne). Nadaj unikalne przypadek_id (np. P-04).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>kroki_przypadku: kroki przypadku w kolejności lp (1, 2, 3...). Wybierz punkt i stan. W co_sie_stalo opisz, co zadziałało lub nie. Punkt, którego przypadek nie dotknął, po prostu pomiń.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Stany kroku (stan)</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>zadzialal, czesciowo, nie_zadzialal, brakuje (punkt, który powinien wystąpić, a go nie było). Etykiety są w zakładce slowniki.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Tory mapy</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Domyślnie wynikają z macierzy i podtypu punktu (importer, dealer, salon, serwis). Nowy tor: wpisz jego nazwę w kolumnie tor_nadpisanie punktu i dodaj etykietę w slowniki (grupa tor; kolejność wierszy to kolejność torów; ID toru nie może być samą liczbą).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>status_danych</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Wartość DEMO oznacza dane przykładowe. Wiersze własne oznacz inaczej albo zostaw puste; nie zostawiaj DEMO przy danych prawdziwych.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Po edycji</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Zapisz plik i zamknij Excela. Kliknij dwukrotnie konwertuj-dane.command (macOS) albo konwertuj-dane.bat (Windows). Jeśli pojawi się błąd, zawiera nazwę zakładki i numer wiersza do poprawy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Zasady</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Nie zmieniaj nazw zakładek ani nagłówków kolumn, nie wstawiaj kolumn ani pustych wierszy w środku tabeli. Teksty wpisuj zwykłym tekstem.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="002E7D32"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -462,72 +647,72 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>macierz</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="5" t="inlineStr">
         <is>
           <t>punkt_styku</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="5" t="inlineStr">
         <is>
           <t>proces</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="5" t="inlineStr">
         <is>
           <t>emocja</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="5" t="inlineStr">
         <is>
           <t>emocja_1_5</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="5" t="inlineStr">
         <is>
           <t>wplyw_na_emocje</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="5" t="inlineStr">
         <is>
           <t>monitoring</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="5" t="inlineStr">
         <is>
           <t>wlasciciel</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" s="5" t="inlineStr">
         <is>
           <t>ocena_cx</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" s="5" t="inlineStr">
         <is>
           <t>status_danych</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" s="5" t="inlineStr">
         <is>
           <t>podtyp</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" s="5" t="inlineStr">
         <is>
           <t>zaopiekowanie_1_5</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" s="5" t="inlineStr">
         <is>
           <t>tor_nadpisanie</t>
         </is>
@@ -559,10 +744,8 @@
           <t>Zainteresowanie</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="F2" s="2" t="n">
+        <v>4</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
@@ -621,10 +804,8 @@
           <t>Ciekawość</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="F3" s="2" t="n">
+        <v>4</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
@@ -683,10 +864,8 @@
           <t>Ekscytacja</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="F4" s="2" t="n">
+        <v>5</v>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
@@ -745,10 +924,8 @@
           <t>Ciekawość</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="F5" s="2" t="n">
+        <v>4</v>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
@@ -807,10 +984,8 @@
           <t>Zaangażowanie</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="F6" s="2" t="n">
+        <v>4</v>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
@@ -869,10 +1044,8 @@
           <t>Irytacja</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="F7" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
@@ -931,10 +1104,8 @@
           <t>Niepewność</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="F8" s="2" t="n">
+        <v>3</v>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
@@ -993,10 +1164,8 @@
           <t>Frustracja</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="F9" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
@@ -1055,10 +1224,8 @@
           <t>Niepewność</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="F10" s="2" t="n">
+        <v>3</v>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
@@ -1165,10 +1332,8 @@
           <t>Napięcie</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="F12" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
@@ -1227,10 +1392,8 @@
           <t>Ulga</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="F13" s="2" t="n">
+        <v>4</v>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
@@ -1289,10 +1452,8 @@
           <t>Niecierpliwość</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="F14" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
@@ -1351,10 +1512,8 @@
           <t>Złość</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="F15" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
@@ -1413,10 +1572,8 @@
           <t>Znużenie</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="F16" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
@@ -1475,10 +1632,8 @@
           <t>Radość</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="F17" s="2" t="n">
+        <v>5</v>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
@@ -1537,10 +1692,8 @@
           <t>Wygoda</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="F18" s="2" t="n">
+        <v>4</v>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
@@ -1599,10 +1752,8 @@
           <t>Obojętność</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="F19" s="2" t="n">
+        <v>3</v>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
@@ -1661,10 +1812,8 @@
           <t>Rozczarowanie</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="F20" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
@@ -1723,10 +1872,8 @@
           <t>Ulga</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="F21" s="2" t="n">
+        <v>4</v>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
@@ -1785,10 +1932,8 @@
           <t>Niepokój</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="F22" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
@@ -1847,10 +1992,8 @@
           <t>Obojętność</t>
         </is>
       </c>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="F23" s="2" t="n">
+        <v>3</v>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
@@ -1909,10 +2052,8 @@
           <t>Napięcie</t>
         </is>
       </c>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="F24" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
@@ -1971,10 +2112,8 @@
           <t>Złość</t>
         </is>
       </c>
-      <c r="F25" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="F25" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
@@ -2033,10 +2172,8 @@
           <t>Zaangażowanie</t>
         </is>
       </c>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="F26" s="2" t="n">
+        <v>3</v>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
@@ -2095,10 +2232,8 @@
           <t>Docenienie</t>
         </is>
       </c>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="F27" s="2" t="n">
+        <v>4</v>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
@@ -2157,10 +2292,8 @@
           <t>Obojętność</t>
         </is>
       </c>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="F28" s="2" t="n">
+        <v>3</v>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
@@ -2219,10 +2352,8 @@
           <t>Duma</t>
         </is>
       </c>
-      <c r="F29" s="2" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="F29" s="2" t="n">
+        <v>5</v>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
@@ -2281,10 +2412,8 @@
           <t>Zainteresowanie</t>
         </is>
       </c>
-      <c r="F30" s="2" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="F30" s="2" t="n">
+        <v>3</v>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
@@ -2343,10 +2472,8 @@
           <t>Niepewność</t>
         </is>
       </c>
-      <c r="F31" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="F31" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
@@ -2405,10 +2532,8 @@
           <t>Oczekiwanie</t>
         </is>
       </c>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="F32" s="2" t="n">
+        <v>3</v>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
@@ -2471,10 +2596,8 @@
           <t>Irytacja</t>
         </is>
       </c>
-      <c r="F33" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="F33" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
@@ -2537,10 +2660,8 @@
           <t>Wygoda</t>
         </is>
       </c>
-      <c r="F34" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="F34" s="2" t="n">
+        <v>4</v>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
@@ -2603,10 +2724,8 @@
           <t>Zaciekawienie</t>
         </is>
       </c>
-      <c r="F35" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="F35" s="2" t="n">
+        <v>4</v>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
@@ -2669,10 +2788,8 @@
           <t>Zaangażowanie</t>
         </is>
       </c>
-      <c r="F36" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="F36" s="2" t="n">
+        <v>4</v>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
@@ -2735,10 +2852,8 @@
           <t>Ekscytacja</t>
         </is>
       </c>
-      <c r="F37" s="2" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="F37" s="2" t="n">
+        <v>5</v>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
@@ -2801,10 +2916,8 @@
           <t>Ekscytacja</t>
         </is>
       </c>
-      <c r="F38" s="2" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="F38" s="2" t="n">
+        <v>5</v>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
@@ -2867,10 +2980,8 @@
           <t>Napięcie</t>
         </is>
       </c>
-      <c r="F39" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="F39" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
@@ -2933,10 +3044,8 @@
           <t>Napięcie</t>
         </is>
       </c>
-      <c r="F40" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="F40" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
@@ -2999,10 +3108,8 @@
           <t>Niepewność</t>
         </is>
       </c>
-      <c r="F41" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="F41" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
@@ -3065,10 +3172,8 @@
           <t>Niepewność</t>
         </is>
       </c>
-      <c r="F42" s="2" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="F42" s="2" t="n">
+        <v>3</v>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
@@ -3131,10 +3236,8 @@
           <t>Znużenie</t>
         </is>
       </c>
-      <c r="F43" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="F43" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
@@ -3197,10 +3300,8 @@
           <t>Oczekiwanie</t>
         </is>
       </c>
-      <c r="F44" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="F44" s="2" t="n">
+        <v>4</v>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
@@ -3263,10 +3364,8 @@
           <t>Radość</t>
         </is>
       </c>
-      <c r="F45" s="2" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="F45" s="2" t="n">
+        <v>5</v>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
@@ -3329,10 +3428,8 @@
           <t>Pewność</t>
         </is>
       </c>
-      <c r="F46" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="F46" s="2" t="n">
+        <v>4</v>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
@@ -3395,10 +3492,8 @@
           <t>Docenienie</t>
         </is>
       </c>
-      <c r="F47" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="F47" s="2" t="n">
+        <v>4</v>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
@@ -3461,10 +3556,8 @@
           <t>Wygoda</t>
         </is>
       </c>
-      <c r="F48" s="2" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="F48" s="2" t="n">
+        <v>3</v>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
@@ -3527,10 +3620,8 @@
           <t>Niepewność</t>
         </is>
       </c>
-      <c r="F49" s="2" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="F49" s="2" t="n">
+        <v>3</v>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
@@ -3593,10 +3684,8 @@
           <t>Niepokój</t>
         </is>
       </c>
-      <c r="F50" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="F50" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
@@ -3659,10 +3748,8 @@
           <t>Złość</t>
         </is>
       </c>
-      <c r="F51" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="F51" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
@@ -3725,10 +3812,8 @@
           <t>Wdzięczność</t>
         </is>
       </c>
-      <c r="F52" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="F52" s="2" t="n">
+        <v>4</v>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
@@ -3791,10 +3876,8 @@
           <t>Znużenie</t>
         </is>
       </c>
-      <c r="F53" s="2" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="F53" s="2" t="n">
+        <v>3</v>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
@@ -3857,10 +3940,8 @@
           <t>Niecierpliwość</t>
         </is>
       </c>
-      <c r="F54" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="F54" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
@@ -3975,10 +4056,8 @@
           <t>Obojętność</t>
         </is>
       </c>
-      <c r="F56" s="2" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="F56" s="2" t="n">
+        <v>3</v>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
@@ -4041,10 +4120,8 @@
           <t>Docenienie</t>
         </is>
       </c>
-      <c r="F57" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="F57" s="2" t="n">
+        <v>4</v>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
@@ -4107,10 +4184,8 @@
           <t>Napięcie</t>
         </is>
       </c>
-      <c r="F58" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="F58" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
@@ -4173,10 +4248,8 @@
           <t>Stres</t>
         </is>
       </c>
-      <c r="F59" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="F59" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
@@ -4239,10 +4312,8 @@
           <t>Nieufność</t>
         </is>
       </c>
-      <c r="F60" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="F60" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
@@ -4305,10 +4376,8 @@
           <t>Zainteresowanie</t>
         </is>
       </c>
-      <c r="F61" s="2" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="F61" s="2" t="n">
+        <v>3</v>
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
@@ -4347,13 +4416,39 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:N61"/>
+  <dataValidations count="7">
+    <dataValidation sqref="A2:A1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Macierz" error="Wybierz wartość z listy (słownik)." type="list">
+      <formula1>=slowniki!$B$2:$B$3</formula1>
+    </dataValidation>
+    <dataValidation sqref="L2:L1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Podtyp" error="Wybierz wartość z listy (słownik) albo zostaw puste." type="list">
+      <formula1>=slowniki!$B$4:$B$6</formula1>
+    </dataValidation>
+    <dataValidation sqref="J2:J1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Ocena CX" error="Wybierz wartość z listy (słownik)." type="list">
+      <formula1>=slowniki!$B$7:$B$10</formula1>
+    </dataValidation>
+    <dataValidation sqref="H2:H1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Monitoring" error="Wybierz wartość z listy (słownik)." type="list">
+      <formula1>=slowniki!$B$11:$B$13</formula1>
+    </dataValidation>
+    <dataValidation sqref="D2:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Proces" error="Wybierz proces z zakładki procesy." type="list">
+      <formula1>=procesy!$B$2:$B$1000</formula1>
+    </dataValidation>
+    <dataValidation sqref="F2:F1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Skala 1-5" error="Wpisz liczbę całkowitą od 1 do 5." type="whole" operator="between">
+      <formula1>1</formula1>
+      <formula2>5</formula2>
+    </dataValidation>
+    <dataValidation sqref="M2:M1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Skala 1-5" error="Wpisz liczbę całkowitą od 1 do 5." type="whole" operator="between">
+      <formula1>1</formula1>
+      <formula2>5</formula2>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="002E7D32"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -4368,27 +4463,27 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>punkt_id</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="5" t="inlineStr">
         <is>
           <t>typ</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="5" t="inlineStr">
         <is>
           <t>tresc</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="5" t="inlineStr">
         <is>
           <t>status_danych</t>
         </is>
@@ -14089,13 +14184,22 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:E360"/>
+  <dataValidations count="2">
+    <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Punkt" error="Wybierz ID z zakładki punkty_styku." type="list">
+      <formula1>=punkty_styku!$B$2:$B$1000</formula1>
+    </dataValidation>
+    <dataValidation sqref="C2:C1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Typ cechy" error="Wybierz wartość z listy (słownik)." type="list">
+      <formula1>=slowniki!$B$14:$B$18</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="002E7D32"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -14115,52 +14219,52 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>punkt_id</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="5" t="inlineStr">
         <is>
           <t>rodzaj</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="5" t="inlineStr">
         <is>
           <t>opis</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="5" t="inlineStr">
         <is>
           <t>koszt</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="5" t="inlineStr">
         <is>
           <t>ryzyko</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="5" t="inlineStr">
         <is>
           <t>zysk</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="5" t="inlineStr">
         <is>
           <t>czas_wdrozenia_tyg</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="5" t="inlineStr">
         <is>
           <t>ryzyka_wdrozenia</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" s="5" t="inlineStr">
         <is>
           <t>status_danych</t>
         </is>
@@ -16918,13 +17022,35 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:J56"/>
+  <dataValidations count="6">
+    <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Punkt" error="Wybierz ID z zakładki punkty_styku." type="list">
+      <formula1>=punkty_styku!$B$2:$B$1000</formula1>
+    </dataValidation>
+    <dataValidation sqref="C2:C1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Rodzaj akcji" error="Wybierz wartość z listy (słownik)." type="list">
+      <formula1>=slowniki!$B$19:$B$20</formula1>
+    </dataValidation>
+    <dataValidation sqref="E2:E1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Koszt" error="Wybierz: niski, średni albo wysoki." type="list">
+      <formula1>"niski,średni,wysoki"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F2:F1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Ryzyko" error="Wybierz: niski, średni albo wysoki." type="list">
+      <formula1>"niski,średni,wysoki"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G2:G1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Zysk" error="Wybierz: niski, średni albo wysoki." type="list">
+      <formula1>"niski,średni,wysoki"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H2:H1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Czas" error="Wpisz liczbę całkowitą tygodni." type="whole" operator="between">
+      <formula1>0</formula1>
+      <formula2>1000</formula2>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="009E9E9E"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -16937,17 +17063,17 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>grupa</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>klucz</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="5" t="inlineStr">
         <is>
           <t>etykieta</t>
         </is>
@@ -17350,9 +17476,10 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="009E9E9E"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -17364,12 +17491,12 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>lp</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>nazwa</t>
         </is>
@@ -17521,9 +17648,10 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="002E7D32"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -17538,27 +17666,27 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>punkt_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>nastepny_id</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="5" t="inlineStr">
         <is>
           <t>etykieta</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="5" t="inlineStr">
         <is>
           <t>opcjonalny</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="5" t="inlineStr">
         <is>
           <t>status_danych</t>
         </is>
@@ -19539,13 +19667,25 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:E84"/>
+  <dataValidations count="3">
+    <dataValidation sqref="A2:A1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Punkt" error="Wybierz ID z zakładki punkty_styku." type="list">
+      <formula1>=punkty_styku!$B$2:$B$1000</formula1>
+    </dataValidation>
+    <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Punkt" error="Wybierz ID z zakładki punkty_styku." type="list">
+      <formula1>=punkty_styku!$B$2:$B$1000</formula1>
+    </dataValidation>
+    <dataValidation sqref="D2:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Opcjonalny" error="Wybierz: tak albo nie (puste = nie)." type="list">
+      <formula1>"tak,nie"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="002E7D32"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -19561,32 +19701,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>przypadek_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>nazwa</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="5" t="inlineStr">
         <is>
           <t>klient</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="5" t="inlineStr">
         <is>
           <t>model_pojazdu</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="5" t="inlineStr">
         <is>
           <t>numer_sprawy</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="5" t="inlineStr">
         <is>
           <t>status_danych</t>
         </is>
@@ -19682,9 +19822,10 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="002E7D32"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -19700,32 +19841,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>przypadek_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>lp</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="5" t="inlineStr">
         <is>
           <t>punkt_id</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="5" t="inlineStr">
         <is>
           <t>stan</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="5" t="inlineStr">
         <is>
           <t>co_sie_stalo</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="5" t="inlineStr">
         <is>
           <t>status_danych</t>
         </is>
@@ -20633,6 +20774,21 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:F31"/>
+  <dataValidations count="4">
+    <dataValidation sqref="A2:A1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Przypadek" error="Wybierz ID z zakładki przypadki." type="list">
+      <formula1>=przypadki!$A$2:$A$1000</formula1>
+    </dataValidation>
+    <dataValidation sqref="C2:C1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Punkt" error="Wybierz ID z zakładki punkty_styku." type="list">
+      <formula1>=punkty_styku!$B$2:$B$1000</formula1>
+    </dataValidation>
+    <dataValidation sqref="D2:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Stan" error="Wybierz wartość z listy (słownik)." type="list">
+      <formula1>=slowniki!$B$21:$B$24</formula1>
+    </dataValidation>
+    <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Numer kroku" error="Wpisz liczbę całkowitą od 1 w górę." type="whole" operator="between">
+      <formula1>1</formula1>
+      <formula2>5</formula2>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Arkusz punkty_styku: kolumna podtyp zaraz obok kolumny macierz
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/macierz-demo.xlsx
+++ b/macierz-demo.xlsx
@@ -632,16 +632,16 @@
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="32" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="46" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="27" customWidth="1" min="9" max="9"/>
-    <col width="17" customWidth="1" min="10" max="10"/>
-    <col width="15" customWidth="1" min="11" max="11"/>
-    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="46" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="27" customWidth="1" min="10" max="10"/>
+    <col width="17" customWidth="1" min="11" max="11"/>
+    <col width="15" customWidth="1" min="12" max="12"/>
     <col width="19" customWidth="1" min="13" max="13"/>
     <col width="16" customWidth="1" min="14" max="14"/>
   </cols>
@@ -654,57 +654,57 @@
       </c>
       <c r="B1" s="5" t="inlineStr">
         <is>
+          <t>podtyp</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
           <t>id</t>
         </is>
       </c>
-      <c r="C1" s="5" t="inlineStr">
+      <c r="D1" s="5" t="inlineStr">
         <is>
           <t>punkt_styku</t>
         </is>
       </c>
-      <c r="D1" s="5" t="inlineStr">
+      <c r="E1" s="5" t="inlineStr">
         <is>
           <t>proces</t>
         </is>
       </c>
-      <c r="E1" s="5" t="inlineStr">
+      <c r="F1" s="5" t="inlineStr">
         <is>
           <t>emocja</t>
         </is>
       </c>
-      <c r="F1" s="5" t="inlineStr">
+      <c r="G1" s="5" t="inlineStr">
         <is>
           <t>emocja_1_5</t>
         </is>
       </c>
-      <c r="G1" s="5" t="inlineStr">
+      <c r="H1" s="5" t="inlineStr">
         <is>
           <t>wplyw_na_emocje</t>
         </is>
       </c>
-      <c r="H1" s="5" t="inlineStr">
+      <c r="I1" s="5" t="inlineStr">
         <is>
           <t>monitoring</t>
         </is>
       </c>
-      <c r="I1" s="5" t="inlineStr">
+      <c r="J1" s="5" t="inlineStr">
         <is>
           <t>wlasciciel</t>
         </is>
       </c>
-      <c r="J1" s="5" t="inlineStr">
+      <c r="K1" s="5" t="inlineStr">
         <is>
           <t>ocena_cx</t>
         </is>
       </c>
-      <c r="K1" s="5" t="inlineStr">
+      <c r="L1" s="5" t="inlineStr">
         <is>
           <t>status_danych</t>
-        </is>
-      </c>
-      <c r="L1" s="5" t="inlineStr">
-        <is>
-          <t>podtyp</t>
         </is>
       </c>
       <c r="M1" s="5" t="inlineStr">
@@ -724,55 +724,55 @@
           <t>importer</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr"/>
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>imp-01</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Reklama TV i radio</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Pozyskanie</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Zainteresowanie</t>
         </is>
       </c>
-      <c r="F2" s="2" t="n">
+      <c r="G2" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Buduje pierwsze skojarzenia z marką</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>tak</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>Marketing importera</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
       <c r="M2" s="2" t="n">
         <v>4</v>
       </c>
@@ -784,55 +784,55 @@
           <t>importer</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr"/>
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>imp-02</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>Media społecznościowe</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>Pozyskanie</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>Ciekawość</t>
         </is>
       </c>
-      <c r="F3" s="2" t="n">
+      <c r="G3" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Daje poczucie bliskości marki</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>częściowo</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>Marketing importera</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>do_poprawy</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="L3" s="2" t="inlineStr"/>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
       <c r="M3" s="2" t="n">
         <v>3</v>
       </c>
@@ -844,55 +844,55 @@
           <t>importer</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr"/>
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>imp-03</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Targi i wydarzenia</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Pozyskanie</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>Ekscytacja</t>
         </is>
       </c>
-      <c r="F4" s="2" t="n">
+      <c r="G4" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>Bezpośredni kontakt z autem i ludźmi</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>nie</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>Marketing importera</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>niezaopiekowany</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="L4" s="2" t="inlineStr"/>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
       <c r="M4" s="2" t="n">
         <v>1</v>
       </c>
@@ -904,55 +904,55 @@
           <t>importer</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr"/>
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>imp-04</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>Strona www marki</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>Pozyskanie</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>Ciekawość</t>
         </is>
       </c>
-      <c r="F5" s="2" t="n">
+      <c r="G5" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>Pierwsze wrażenie o marce i ofercie</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>tak</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>E-commerce importera</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>do_poprawy</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="L5" s="2" t="inlineStr"/>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
       <c r="M5" s="2" t="n">
         <v>3</v>
       </c>
@@ -964,55 +964,55 @@
           <t>importer</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr"/>
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>imp-05</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>Konfigurator online</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>Zakup</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Zaangażowanie</t>
         </is>
       </c>
-      <c r="F6" s="2" t="n">
+      <c r="G6" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>Daje poczucie kontroli i personalizacji</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>częściowo</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>E-commerce importera</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>do_poprawy</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="L6" s="2" t="inlineStr"/>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
       <c r="M6" s="2" t="n">
         <v>3</v>
       </c>
@@ -1024,55 +1024,55 @@
           <t>importer</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr"/>
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>imp-06</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>Wyszukiwarka dealerów</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>Zakup</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Irytacja</t>
         </is>
       </c>
-      <c r="F7" s="2" t="n">
+      <c r="G7" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>Błędne dane utrudniają pierwszy kontakt</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>nie</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>Sprzedaż importera</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>niezaopiekowany</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="L7" s="2" t="inlineStr"/>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
       <c r="M7" s="2" t="n">
         <v>2</v>
       </c>
@@ -1084,55 +1084,55 @@
           <t>importer</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr"/>
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>imp-07</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>Infolinia sprzedażowa</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>Zakup</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Niepewność</t>
         </is>
       </c>
-      <c r="F8" s="2" t="n">
+      <c r="G8" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>Rozmowa daje lub odbiera pewność wyboru</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>tak</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>Obsługa klienta importera</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>do_poprawy</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="L8" s="2" t="inlineStr"/>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
       <c r="M8" s="2" t="n">
         <v>3</v>
       </c>
@@ -1144,55 +1144,55 @@
           <t>importer</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr"/>
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>imp-08</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>Czat i chatbot</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>Zakup</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>Frustracja</t>
         </is>
       </c>
-      <c r="F9" s="2" t="n">
+      <c r="G9" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>Brak zrozumienia pytań obniża nastrój</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>tak</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>Obsługa klienta importera</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>do_poprawy</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="L9" s="2" t="inlineStr"/>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
       <c r="M9" s="2" t="n">
         <v>3</v>
       </c>
@@ -1204,55 +1204,55 @@
           <t>importer</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr"/>
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>imp-09</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>Kalkulator finansowania</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>Finansowanie</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>Niepewność</t>
         </is>
       </c>
-      <c r="F10" s="2" t="n">
+      <c r="G10" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>Pomaga lub zniechęca do zakupu</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>częściowo</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>Finanse importera</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>do_poprawy</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="L10" s="2" t="inlineStr"/>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
       <c r="M10" s="2" t="n">
         <v>3</v>
       </c>
@@ -1264,45 +1264,45 @@
           <t>importer</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr"/>
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>imp-10</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>Ubezpieczenie w pakiecie</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>Finansowanie</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr"/>
       <c r="G11" s="2" t="inlineStr"/>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>nie</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>Finanse importera</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>brak_oceny</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="L11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
       <c r="M11" s="2" t="inlineStr"/>
       <c r="N11" s="2" t="inlineStr"/>
     </row>
@@ -1312,55 +1312,55 @@
           <t>importer</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr"/>
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>imp-11</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>Wniosek o finansowanie</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>Finansowanie</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>Napięcie</t>
         </is>
       </c>
-      <c r="F12" s="2" t="n">
+      <c r="G12" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>Czekanie na decyzję budzi stres</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>tak</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>Finanse importera</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>do_poprawy</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="L12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
       <c r="M12" s="2" t="n">
         <v>3</v>
       </c>
@@ -1372,55 +1372,55 @@
           <t>importer</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr"/>
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>imp-12</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>Potwierdzenie zamówienia</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>Zamówienie</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>Ulga</t>
         </is>
       </c>
-      <c r="F13" s="2" t="n">
+      <c r="G13" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>Daje poczucie bezpieczeństwa</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>tak</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="J13" s="2" t="inlineStr">
         <is>
           <t>Logistyka importera</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr">
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="K13" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="L13" s="2" t="inlineStr"/>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
       <c r="M13" s="2" t="n">
         <v>5</v>
       </c>
@@ -1432,55 +1432,55 @@
           <t>importer</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr"/>
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>imp-13</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>Status produkcji i dostawy</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>Zamówienie</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>Niecierpliwość</t>
         </is>
       </c>
-      <c r="F14" s="2" t="n">
+      <c r="G14" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>Brak informacji wydłuża oczekiwanie</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="I14" s="2" t="inlineStr">
         <is>
           <t>nie</t>
         </is>
       </c>
-      <c r="I14" s="2" t="inlineStr">
+      <c r="J14" s="2" t="inlineStr">
         <is>
           <t>Logistyka importera</t>
         </is>
       </c>
-      <c r="J14" s="2" t="inlineStr">
+      <c r="K14" s="2" t="inlineStr">
         <is>
           <t>niezaopiekowany</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="L14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
       <c r="M14" s="2" t="n">
         <v>1</v>
       </c>
@@ -1492,55 +1492,55 @@
           <t>importer</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr"/>
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>imp-14</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>Opóźnienie dostawy</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>Zamówienie</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="F15" s="2" t="inlineStr">
         <is>
           <t>Złość</t>
         </is>
       </c>
-      <c r="F15" s="2" t="n">
+      <c r="G15" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="H15" s="2" t="inlineStr">
         <is>
           <t>Zerwanie obietnicy mocno obniża zaufanie</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="I15" s="2" t="inlineStr">
         <is>
           <t>tak</t>
         </is>
       </c>
-      <c r="I15" s="2" t="inlineStr">
+      <c r="J15" s="2" t="inlineStr">
         <is>
           <t>Logistyka importera</t>
         </is>
       </c>
-      <c r="J15" s="2" t="inlineStr">
+      <c r="K15" s="2" t="inlineStr">
         <is>
           <t>do_poprawy</t>
         </is>
       </c>
-      <c r="K15" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="L15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
       <c r="M15" s="2" t="n">
         <v>3</v>
       </c>
@@ -1552,55 +1552,55 @@
           <t>importer</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr"/>
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>imp-15</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>Rejestracja i dokumenty</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>Dostawa</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>Znużenie</t>
         </is>
       </c>
-      <c r="F16" s="2" t="n">
+      <c r="G16" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>Formalności psują radość z zakupu</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="I16" s="2" t="inlineStr">
         <is>
           <t>nie</t>
         </is>
       </c>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="J16" s="2" t="inlineStr">
         <is>
           <t>Sprzedaż importera</t>
         </is>
       </c>
-      <c r="J16" s="2" t="inlineStr">
+      <c r="K16" s="2" t="inlineStr">
         <is>
           <t>niezaopiekowany</t>
         </is>
       </c>
-      <c r="K16" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="L16" s="2" t="inlineStr"/>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
       <c r="M16" s="2" t="n">
         <v>2</v>
       </c>
@@ -1612,55 +1612,55 @@
           <t>importer</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr"/>
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>imp-16</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>Pakiet powitalny</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>Dostawa</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t>Radość</t>
         </is>
       </c>
-      <c r="F17" s="2" t="n">
+      <c r="G17" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="H17" s="2" t="inlineStr">
         <is>
           <t>Wzmacnia emocje zakupu</t>
         </is>
       </c>
-      <c r="H17" s="2" t="inlineStr">
+      <c r="I17" s="2" t="inlineStr">
         <is>
           <t>częściowo</t>
         </is>
       </c>
-      <c r="I17" s="2" t="inlineStr">
+      <c r="J17" s="2" t="inlineStr">
         <is>
           <t>Marketing importera</t>
         </is>
       </c>
-      <c r="J17" s="2" t="inlineStr">
+      <c r="K17" s="2" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="K17" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="L17" s="2" t="inlineStr"/>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
       <c r="M17" s="2" t="n">
         <v>4</v>
       </c>
@@ -1672,55 +1672,55 @@
           <t>importer</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr"/>
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>imp-17</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>Aplikacja mobilna</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>Użytkowanie</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>Wygoda</t>
         </is>
       </c>
-      <c r="F18" s="2" t="n">
+      <c r="G18" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>Ułatwia codzienne korzystanie</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr">
+      <c r="I18" s="2" t="inlineStr">
         <is>
           <t>tak</t>
         </is>
       </c>
-      <c r="I18" s="2" t="inlineStr">
+      <c r="J18" s="2" t="inlineStr">
         <is>
           <t>Produkt i usługi cyfrowe</t>
         </is>
       </c>
-      <c r="J18" s="2" t="inlineStr">
+      <c r="K18" s="2" t="inlineStr">
         <is>
           <t>do_poprawy</t>
         </is>
       </c>
-      <c r="K18" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="L18" s="2" t="inlineStr"/>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
       <c r="M18" s="2" t="n">
         <v>3</v>
       </c>
@@ -1732,55 +1732,55 @@
           <t>importer</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr"/>
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>imp-18</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>Aktualizacje oprogramowania</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr">
         <is>
           <t>Użytkowanie</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="F19" s="2" t="inlineStr">
         <is>
           <t>Obojętność</t>
         </is>
       </c>
-      <c r="F19" s="2" t="n">
+      <c r="G19" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G19" s="2" t="inlineStr">
+      <c r="H19" s="2" t="inlineStr">
         <is>
           <t>Neutralne gdy działają, irytują gdy zawodzą</t>
         </is>
       </c>
-      <c r="H19" s="2" t="inlineStr">
+      <c r="I19" s="2" t="inlineStr">
         <is>
           <t>częściowo</t>
         </is>
       </c>
-      <c r="I19" s="2" t="inlineStr">
+      <c r="J19" s="2" t="inlineStr">
         <is>
           <t>Produkt i usługi cyfrowe</t>
         </is>
       </c>
-      <c r="J19" s="2" t="inlineStr">
+      <c r="K19" s="2" t="inlineStr">
         <is>
           <t>do_poprawy</t>
         </is>
       </c>
-      <c r="K19" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="L19" s="2" t="inlineStr"/>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
       <c r="M19" s="2" t="n">
         <v>3</v>
       </c>
@@ -1792,55 +1792,55 @@
           <t>importer</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr"/>
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>imp-19</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>Usługi łączności (Connected)</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>Użytkowanie</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>Rozczarowanie</t>
         </is>
       </c>
-      <c r="F20" s="2" t="n">
+      <c r="G20" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="H20" s="2" t="inlineStr">
         <is>
           <t>Niespełnione obietnice cyfrowe</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr">
+      <c r="I20" s="2" t="inlineStr">
         <is>
           <t>nie</t>
         </is>
       </c>
-      <c r="I20" s="2" t="inlineStr">
+      <c r="J20" s="2" t="inlineStr">
         <is>
           <t>Produkt i usługi cyfrowe</t>
         </is>
       </c>
-      <c r="J20" s="2" t="inlineStr">
+      <c r="K20" s="2" t="inlineStr">
         <is>
           <t>niezaopiekowany</t>
         </is>
       </c>
-      <c r="K20" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="L20" s="2" t="inlineStr"/>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
       <c r="M20" s="2" t="n">
         <v>1</v>
       </c>
@@ -1852,55 +1852,55 @@
           <t>importer</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr"/>
+      <c r="C21" s="2" t="inlineStr">
         <is>
           <t>imp-20</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>Pomoc drogowa</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>Użytkowanie</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="F21" s="2" t="inlineStr">
         <is>
           <t>Ulga</t>
         </is>
       </c>
-      <c r="F21" s="2" t="n">
+      <c r="G21" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G21" s="2" t="inlineStr">
+      <c r="H21" s="2" t="inlineStr">
         <is>
           <t>W kryzysie liczy się szybkość i empatia</t>
         </is>
       </c>
-      <c r="H21" s="2" t="inlineStr">
+      <c r="I21" s="2" t="inlineStr">
         <is>
           <t>tak</t>
         </is>
       </c>
-      <c r="I21" s="2" t="inlineStr">
+      <c r="J21" s="2" t="inlineStr">
         <is>
           <t>Obsługa klienta importera</t>
         </is>
       </c>
-      <c r="J21" s="2" t="inlineStr">
+      <c r="K21" s="2" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="K21" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="L21" s="2" t="inlineStr"/>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
       <c r="M21" s="2" t="n">
         <v>5</v>
       </c>
@@ -1912,55 +1912,55 @@
           <t>importer</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr"/>
+      <c r="C22" s="2" t="inlineStr">
         <is>
           <t>imp-21</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>Kampania serwisowa</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr">
+      <c r="E22" s="2" t="inlineStr">
         <is>
           <t>Posprzedaż</t>
         </is>
       </c>
-      <c r="E22" s="2" t="inlineStr">
+      <c r="F22" s="2" t="inlineStr">
         <is>
           <t>Niepokój</t>
         </is>
       </c>
-      <c r="F22" s="2" t="n">
+      <c r="G22" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="H22" s="2" t="inlineStr">
         <is>
           <t>Komunikat o usterce budzi obawy</t>
         </is>
       </c>
-      <c r="H22" s="2" t="inlineStr">
+      <c r="I22" s="2" t="inlineStr">
         <is>
           <t>częściowo</t>
         </is>
       </c>
-      <c r="I22" s="2" t="inlineStr">
+      <c r="J22" s="2" t="inlineStr">
         <is>
           <t>Jakość importera</t>
         </is>
       </c>
-      <c r="J22" s="2" t="inlineStr">
+      <c r="K22" s="2" t="inlineStr">
         <is>
           <t>niezaopiekowany</t>
         </is>
       </c>
-      <c r="K22" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="L22" s="2" t="inlineStr"/>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
       <c r="M22" s="2" t="n">
         <v>2</v>
       </c>
@@ -1972,55 +1972,55 @@
           <t>importer</t>
         </is>
       </c>
-      <c r="B23" s="2" t="inlineStr">
+      <c r="B23" s="2" t="inlineStr"/>
+      <c r="C23" s="2" t="inlineStr">
         <is>
           <t>imp-22</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr">
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t>Przypomnienie o przeglądzie</t>
         </is>
       </c>
-      <c r="D23" s="2" t="inlineStr">
+      <c r="E23" s="2" t="inlineStr">
         <is>
           <t>Posprzedaż</t>
         </is>
       </c>
-      <c r="E23" s="2" t="inlineStr">
+      <c r="F23" s="2" t="inlineStr">
         <is>
           <t>Obojętność</t>
         </is>
       </c>
-      <c r="F23" s="2" t="n">
+      <c r="G23" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G23" s="2" t="inlineStr">
+      <c r="H23" s="2" t="inlineStr">
         <is>
           <t>Rzadko wzbudza emocje</t>
         </is>
       </c>
-      <c r="H23" s="2" t="inlineStr">
+      <c r="I23" s="2" t="inlineStr">
         <is>
           <t>tak</t>
         </is>
       </c>
-      <c r="I23" s="2" t="inlineStr">
+      <c r="J23" s="2" t="inlineStr">
         <is>
           <t>Posprzedaż importera</t>
         </is>
       </c>
-      <c r="J23" s="2" t="inlineStr">
+      <c r="K23" s="2" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="K23" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="L23" s="2" t="inlineStr"/>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
       <c r="M23" s="2" t="n">
         <v>4</v>
       </c>
@@ -2032,55 +2032,55 @@
           <t>importer</t>
         </is>
       </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr"/>
+      <c r="C24" s="2" t="inlineStr">
         <is>
           <t>imp-23</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>Gwarancja i roszczenia</t>
         </is>
       </c>
-      <c r="D24" s="2" t="inlineStr">
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>Posprzedaż</t>
         </is>
       </c>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="F24" s="2" t="inlineStr">
         <is>
           <t>Napięcie</t>
         </is>
       </c>
-      <c r="F24" s="2" t="n">
+      <c r="G24" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="G24" s="2" t="inlineStr">
+      <c r="H24" s="2" t="inlineStr">
         <is>
           <t>Spór o gwarancję mocno obniża zaufanie</t>
         </is>
       </c>
-      <c r="H24" s="2" t="inlineStr">
+      <c r="I24" s="2" t="inlineStr">
         <is>
           <t>tak</t>
         </is>
       </c>
-      <c r="I24" s="2" t="inlineStr">
+      <c r="J24" s="2" t="inlineStr">
         <is>
           <t>Jakość importera</t>
         </is>
       </c>
-      <c r="J24" s="2" t="inlineStr">
+      <c r="K24" s="2" t="inlineStr">
         <is>
           <t>do_poprawy</t>
         </is>
       </c>
-      <c r="K24" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="L24" s="2" t="inlineStr"/>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
       <c r="M24" s="2" t="n">
         <v>3</v>
       </c>
@@ -2092,55 +2092,55 @@
           <t>importer</t>
         </is>
       </c>
-      <c r="B25" s="2" t="inlineStr">
+      <c r="B25" s="2" t="inlineStr"/>
+      <c r="C25" s="2" t="inlineStr">
         <is>
           <t>imp-24</t>
         </is>
       </c>
-      <c r="C25" s="2" t="inlineStr">
+      <c r="D25" s="2" t="inlineStr">
         <is>
           <t>Reklamacje</t>
         </is>
       </c>
-      <c r="D25" s="2" t="inlineStr">
+      <c r="E25" s="2" t="inlineStr">
         <is>
           <t>Reklamacje</t>
         </is>
       </c>
-      <c r="E25" s="2" t="inlineStr">
+      <c r="F25" s="2" t="inlineStr">
         <is>
           <t>Złość</t>
         </is>
       </c>
-      <c r="F25" s="2" t="n">
+      <c r="G25" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="G25" s="2" t="inlineStr">
+      <c r="H25" s="2" t="inlineStr">
         <is>
           <t>Kontakt w sprawie wady budzi silne emocje</t>
         </is>
       </c>
-      <c r="H25" s="2" t="inlineStr">
+      <c r="I25" s="2" t="inlineStr">
         <is>
           <t>tak</t>
         </is>
       </c>
-      <c r="I25" s="2" t="inlineStr">
+      <c r="J25" s="2" t="inlineStr">
         <is>
           <t>Obsługa klienta importera</t>
         </is>
       </c>
-      <c r="J25" s="2" t="inlineStr">
+      <c r="K25" s="2" t="inlineStr">
         <is>
           <t>niezaopiekowany</t>
         </is>
       </c>
-      <c r="K25" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="L25" s="2" t="inlineStr"/>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
       <c r="M25" s="2" t="n">
         <v>1</v>
       </c>
@@ -2152,55 +2152,55 @@
           <t>importer</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr"/>
+      <c r="C26" s="2" t="inlineStr">
         <is>
           <t>imp-25</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
+      <c r="D26" s="2" t="inlineStr">
         <is>
           <t>Ankieta po zakupie</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="E26" s="2" t="inlineStr">
         <is>
           <t>Posprzedaż</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>Zaangażowanie</t>
         </is>
       </c>
-      <c r="F26" s="2" t="n">
+      <c r="G26" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="H26" s="2" t="inlineStr">
         <is>
           <t>Pokazuje że opinia się liczy</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr">
+      <c r="I26" s="2" t="inlineStr">
         <is>
           <t>tak</t>
         </is>
       </c>
-      <c r="I26" s="2" t="inlineStr">
+      <c r="J26" s="2" t="inlineStr">
         <is>
           <t>Badania importera</t>
         </is>
       </c>
-      <c r="J26" s="2" t="inlineStr">
+      <c r="K26" s="2" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="K26" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="L26" s="2" t="inlineStr"/>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
       <c r="M26" s="2" t="n">
         <v>5</v>
       </c>
@@ -2212,55 +2212,55 @@
           <t>importer</t>
         </is>
       </c>
-      <c r="B27" s="2" t="inlineStr">
+      <c r="B27" s="2" t="inlineStr"/>
+      <c r="C27" s="2" t="inlineStr">
         <is>
           <t>imp-26</t>
         </is>
       </c>
-      <c r="C27" s="2" t="inlineStr">
+      <c r="D27" s="2" t="inlineStr">
         <is>
           <t>Program lojalnościowy</t>
         </is>
       </c>
-      <c r="D27" s="2" t="inlineStr">
+      <c r="E27" s="2" t="inlineStr">
         <is>
           <t>Lojalność</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr">
+      <c r="F27" s="2" t="inlineStr">
         <is>
           <t>Docenienie</t>
         </is>
       </c>
-      <c r="F27" s="2" t="n">
+      <c r="G27" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G27" s="2" t="inlineStr">
+      <c r="H27" s="2" t="inlineStr">
         <is>
           <t>Buduje poczucie bycia wyróżnionym</t>
         </is>
       </c>
-      <c r="H27" s="2" t="inlineStr">
+      <c r="I27" s="2" t="inlineStr">
         <is>
           <t>częściowo</t>
         </is>
       </c>
-      <c r="I27" s="2" t="inlineStr">
+      <c r="J27" s="2" t="inlineStr">
         <is>
           <t>CRM importera</t>
         </is>
       </c>
-      <c r="J27" s="2" t="inlineStr">
+      <c r="K27" s="2" t="inlineStr">
         <is>
           <t>do_poprawy</t>
         </is>
       </c>
-      <c r="K27" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="L27" s="2" t="inlineStr"/>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
       <c r="M27" s="2" t="n">
         <v>3</v>
       </c>
@@ -2272,55 +2272,55 @@
           <t>importer</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr"/>
+      <c r="C28" s="2" t="inlineStr">
         <is>
           <t>imp-27</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr">
+      <c r="D28" s="2" t="inlineStr">
         <is>
           <t>Newsletter</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr">
+      <c r="E28" s="2" t="inlineStr">
         <is>
           <t>Lojalność</t>
         </is>
       </c>
-      <c r="E28" s="2" t="inlineStr">
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>Obojętność</t>
         </is>
       </c>
-      <c r="F28" s="2" t="n">
+      <c r="G28" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G28" s="2" t="inlineStr">
+      <c r="H28" s="2" t="inlineStr">
         <is>
           <t>Rzadko wzbudza emocje</t>
         </is>
       </c>
-      <c r="H28" s="2" t="inlineStr">
+      <c r="I28" s="2" t="inlineStr">
         <is>
           <t>tak</t>
         </is>
       </c>
-      <c r="I28" s="2" t="inlineStr">
+      <c r="J28" s="2" t="inlineStr">
         <is>
           <t>CRM importera</t>
         </is>
       </c>
-      <c r="J28" s="2" t="inlineStr">
+      <c r="K28" s="2" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="K28" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="L28" s="2" t="inlineStr"/>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
       <c r="M28" s="2" t="n">
         <v>4</v>
       </c>
@@ -2332,55 +2332,55 @@
           <t>importer</t>
         </is>
       </c>
-      <c r="B29" s="2" t="inlineStr">
+      <c r="B29" s="2" t="inlineStr"/>
+      <c r="C29" s="2" t="inlineStr">
         <is>
           <t>imp-28</t>
         </is>
       </c>
-      <c r="C29" s="2" t="inlineStr">
+      <c r="D29" s="2" t="inlineStr">
         <is>
           <t>Klub właścicieli</t>
         </is>
       </c>
-      <c r="D29" s="2" t="inlineStr">
+      <c r="E29" s="2" t="inlineStr">
         <is>
           <t>Lojalność</t>
         </is>
       </c>
-      <c r="E29" s="2" t="inlineStr">
+      <c r="F29" s="2" t="inlineStr">
         <is>
           <t>Duma</t>
         </is>
       </c>
-      <c r="F29" s="2" t="n">
+      <c r="G29" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="G29" s="2" t="inlineStr">
+      <c r="H29" s="2" t="inlineStr">
         <is>
           <t>Buduje przynależność do marki</t>
         </is>
       </c>
-      <c r="H29" s="2" t="inlineStr">
+      <c r="I29" s="2" t="inlineStr">
         <is>
           <t>nie</t>
         </is>
       </c>
-      <c r="I29" s="2" t="inlineStr">
+      <c r="J29" s="2" t="inlineStr">
         <is>
           <t>Marketing importera</t>
         </is>
       </c>
-      <c r="J29" s="2" t="inlineStr">
+      <c r="K29" s="2" t="inlineStr">
         <is>
           <t>niezaopiekowany</t>
         </is>
       </c>
-      <c r="K29" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="L29" s="2" t="inlineStr"/>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
       <c r="M29" s="2" t="n">
         <v>2</v>
       </c>
@@ -2392,55 +2392,55 @@
           <t>importer</t>
         </is>
       </c>
-      <c r="B30" s="2" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr"/>
+      <c r="C30" s="2" t="inlineStr">
         <is>
           <t>imp-29</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr">
+      <c r="D30" s="2" t="inlineStr">
         <is>
           <t>Oferta wymiany i odkupu</t>
         </is>
       </c>
-      <c r="D30" s="2" t="inlineStr">
+      <c r="E30" s="2" t="inlineStr">
         <is>
           <t>Wymiana</t>
         </is>
       </c>
-      <c r="E30" s="2" t="inlineStr">
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>Zainteresowanie</t>
         </is>
       </c>
-      <c r="F30" s="2" t="n">
+      <c r="G30" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G30" s="2" t="inlineStr">
+      <c r="H30" s="2" t="inlineStr">
         <is>
           <t>Ułatwia decyzję o następnym aucie</t>
         </is>
       </c>
-      <c r="H30" s="2" t="inlineStr">
+      <c r="I30" s="2" t="inlineStr">
         <is>
           <t>nie</t>
         </is>
       </c>
-      <c r="I30" s="2" t="inlineStr">
+      <c r="J30" s="2" t="inlineStr">
         <is>
           <t>Sprzedaż importera</t>
         </is>
       </c>
-      <c r="J30" s="2" t="inlineStr">
+      <c r="K30" s="2" t="inlineStr">
         <is>
           <t>niezaopiekowany</t>
         </is>
       </c>
-      <c r="K30" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="L30" s="2" t="inlineStr"/>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
       <c r="M30" s="2" t="n">
         <v>1</v>
       </c>
@@ -2452,55 +2452,55 @@
           <t>importer</t>
         </is>
       </c>
-      <c r="B31" s="2" t="inlineStr">
+      <c r="B31" s="2" t="inlineStr"/>
+      <c r="C31" s="2" t="inlineStr">
         <is>
           <t>imp-30</t>
         </is>
       </c>
-      <c r="C31" s="2" t="inlineStr">
+      <c r="D31" s="2" t="inlineStr">
         <is>
           <t>Zakończenie umowy leasingu</t>
         </is>
       </c>
-      <c r="D31" s="2" t="inlineStr">
+      <c r="E31" s="2" t="inlineStr">
         <is>
           <t>Wymiana</t>
         </is>
       </c>
-      <c r="E31" s="2" t="inlineStr">
+      <c r="F31" s="2" t="inlineStr">
         <is>
           <t>Niepewność</t>
         </is>
       </c>
-      <c r="F31" s="2" t="n">
+      <c r="G31" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="G31" s="2" t="inlineStr">
+      <c r="H31" s="2" t="inlineStr">
         <is>
           <t>Brak jasnych kroków budzi stres</t>
         </is>
       </c>
-      <c r="H31" s="2" t="inlineStr">
+      <c r="I31" s="2" t="inlineStr">
         <is>
           <t>nie</t>
         </is>
       </c>
-      <c r="I31" s="2" t="inlineStr">
+      <c r="J31" s="2" t="inlineStr">
         <is>
           <t>Finanse importera</t>
         </is>
       </c>
-      <c r="J31" s="2" t="inlineStr">
+      <c r="K31" s="2" t="inlineStr">
         <is>
           <t>do_poprawy</t>
         </is>
       </c>
-      <c r="K31" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="L31" s="2" t="inlineStr"/>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
       <c r="M31" s="2" t="n">
         <v>3</v>
       </c>
@@ -2514,55 +2514,55 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
+          <t>dealer</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
           <t>dea-01</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr">
+      <c r="D32" s="2" t="inlineStr">
         <is>
           <t>Zapytanie przez formularz</t>
         </is>
       </c>
-      <c r="D32" s="2" t="inlineStr">
+      <c r="E32" s="2" t="inlineStr">
         <is>
           <t>Zapytanie</t>
         </is>
       </c>
-      <c r="E32" s="2" t="inlineStr">
+      <c r="F32" s="2" t="inlineStr">
         <is>
           <t>Oczekiwanie</t>
         </is>
       </c>
-      <c r="F32" s="2" t="n">
+      <c r="G32" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G32" s="2" t="inlineStr">
+      <c r="H32" s="2" t="inlineStr">
         <is>
           <t>Szybka odpowiedź buduje zaufanie</t>
         </is>
       </c>
-      <c r="H32" s="2" t="inlineStr">
+      <c r="I32" s="2" t="inlineStr">
         <is>
           <t>tak</t>
         </is>
       </c>
-      <c r="I32" s="2" t="inlineStr">
+      <c r="J32" s="2" t="inlineStr">
         <is>
           <t>Dealer</t>
         </is>
       </c>
-      <c r="J32" s="2" t="inlineStr">
+      <c r="K32" s="2" t="inlineStr">
         <is>
           <t>do_poprawy</t>
         </is>
       </c>
-      <c r="K32" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
       <c r="L32" s="2" t="inlineStr">
         <is>
-          <t>dealer</t>
+          <t>DEMO</t>
         </is>
       </c>
       <c r="M32" s="2" t="n">
@@ -2578,55 +2578,55 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
+          <t>salon</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
           <t>dea-02</t>
         </is>
       </c>
-      <c r="C33" s="2" t="inlineStr">
+      <c r="D33" s="2" t="inlineStr">
         <is>
           <t>Telefon do salonu</t>
         </is>
       </c>
-      <c r="D33" s="2" t="inlineStr">
+      <c r="E33" s="2" t="inlineStr">
         <is>
           <t>Zapytanie</t>
         </is>
       </c>
-      <c r="E33" s="2" t="inlineStr">
+      <c r="F33" s="2" t="inlineStr">
         <is>
           <t>Irytacja</t>
         </is>
       </c>
-      <c r="F33" s="2" t="n">
+      <c r="G33" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="G33" s="2" t="inlineStr">
+      <c r="H33" s="2" t="inlineStr">
         <is>
           <t>Długie oczekiwanie obniża nastrój</t>
         </is>
       </c>
-      <c r="H33" s="2" t="inlineStr">
+      <c r="I33" s="2" t="inlineStr">
         <is>
           <t>nie</t>
         </is>
       </c>
-      <c r="I33" s="2" t="inlineStr">
+      <c r="J33" s="2" t="inlineStr">
         <is>
           <t>Dealer</t>
         </is>
       </c>
-      <c r="J33" s="2" t="inlineStr">
+      <c r="K33" s="2" t="inlineStr">
         <is>
           <t>niezaopiekowany</t>
         </is>
       </c>
-      <c r="K33" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>salon</t>
+          <t>DEMO</t>
         </is>
       </c>
       <c r="M33" s="2" t="n">
@@ -2642,55 +2642,55 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
+          <t>salon</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
           <t>dea-03</t>
         </is>
       </c>
-      <c r="C34" s="2" t="inlineStr">
+      <c r="D34" s="2" t="inlineStr">
         <is>
           <t>Czat i WhatsApp salonu</t>
         </is>
       </c>
-      <c r="D34" s="2" t="inlineStr">
+      <c r="E34" s="2" t="inlineStr">
         <is>
           <t>Zapytanie</t>
         </is>
       </c>
-      <c r="E34" s="2" t="inlineStr">
+      <c r="F34" s="2" t="inlineStr">
         <is>
           <t>Wygoda</t>
         </is>
       </c>
-      <c r="F34" s="2" t="n">
+      <c r="G34" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G34" s="2" t="inlineStr">
+      <c r="H34" s="2" t="inlineStr">
         <is>
           <t>Szybki i wygodny kontakt</t>
         </is>
       </c>
-      <c r="H34" s="2" t="inlineStr">
+      <c r="I34" s="2" t="inlineStr">
         <is>
           <t>częściowo</t>
         </is>
       </c>
-      <c r="I34" s="2" t="inlineStr">
+      <c r="J34" s="2" t="inlineStr">
         <is>
           <t>Dealer</t>
         </is>
       </c>
-      <c r="J34" s="2" t="inlineStr">
+      <c r="K34" s="2" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="K34" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
       <c r="L34" s="2" t="inlineStr">
         <is>
-          <t>salon</t>
+          <t>DEMO</t>
         </is>
       </c>
       <c r="M34" s="2" t="n">
@@ -2706,55 +2706,55 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
+          <t>salon</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
           <t>dea-04</t>
         </is>
       </c>
-      <c r="C35" s="2" t="inlineStr">
+      <c r="D35" s="2" t="inlineStr">
         <is>
           <t>Powitanie w salonie</t>
         </is>
       </c>
-      <c r="D35" s="2" t="inlineStr">
+      <c r="E35" s="2" t="inlineStr">
         <is>
           <t>Zakup</t>
         </is>
       </c>
-      <c r="E35" s="2" t="inlineStr">
+      <c r="F35" s="2" t="inlineStr">
         <is>
           <t>Zaciekawienie</t>
         </is>
       </c>
-      <c r="F35" s="2" t="n">
+      <c r="G35" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G35" s="2" t="inlineStr">
+      <c r="H35" s="2" t="inlineStr">
         <is>
           <t>Atmosfera buduje emocje</t>
         </is>
       </c>
-      <c r="H35" s="2" t="inlineStr">
+      <c r="I35" s="2" t="inlineStr">
         <is>
           <t>nie</t>
         </is>
       </c>
-      <c r="I35" s="2" t="inlineStr">
+      <c r="J35" s="2" t="inlineStr">
         <is>
           <t>Dyrektor salonu</t>
         </is>
       </c>
-      <c r="J35" s="2" t="inlineStr">
+      <c r="K35" s="2" t="inlineStr">
         <is>
           <t>niezaopiekowany</t>
         </is>
       </c>
-      <c r="K35" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
       <c r="L35" s="2" t="inlineStr">
         <is>
-          <t>salon</t>
+          <t>DEMO</t>
         </is>
       </c>
       <c r="M35" s="2" t="n">
@@ -2770,55 +2770,55 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
+          <t>salon</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
           <t>dea-05</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr">
+      <c r="D36" s="2" t="inlineStr">
         <is>
           <t>Analiza potrzeb</t>
         </is>
       </c>
-      <c r="D36" s="2" t="inlineStr">
+      <c r="E36" s="2" t="inlineStr">
         <is>
           <t>Zakup</t>
         </is>
       </c>
-      <c r="E36" s="2" t="inlineStr">
+      <c r="F36" s="2" t="inlineStr">
         <is>
           <t>Zaangażowanie</t>
         </is>
       </c>
-      <c r="F36" s="2" t="n">
+      <c r="G36" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G36" s="2" t="inlineStr">
+      <c r="H36" s="2" t="inlineStr">
         <is>
           <t>Poczucie że doradca słucha</t>
         </is>
       </c>
-      <c r="H36" s="2" t="inlineStr">
+      <c r="I36" s="2" t="inlineStr">
         <is>
           <t>tak</t>
         </is>
       </c>
-      <c r="I36" s="2" t="inlineStr">
+      <c r="J36" s="2" t="inlineStr">
         <is>
           <t>Sprzedaż dealera</t>
         </is>
       </c>
-      <c r="J36" s="2" t="inlineStr">
+      <c r="K36" s="2" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="K36" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
       <c r="L36" s="2" t="inlineStr">
         <is>
-          <t>salon</t>
+          <t>DEMO</t>
         </is>
       </c>
       <c r="M36" s="2" t="n">
@@ -2834,55 +2834,55 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
+          <t>salon</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
           <t>dea-06</t>
         </is>
       </c>
-      <c r="C37" s="2" t="inlineStr">
+      <c r="D37" s="2" t="inlineStr">
         <is>
           <t>Prezentacja auta</t>
         </is>
       </c>
-      <c r="D37" s="2" t="inlineStr">
+      <c r="E37" s="2" t="inlineStr">
         <is>
           <t>Zakup</t>
         </is>
       </c>
-      <c r="E37" s="2" t="inlineStr">
+      <c r="F37" s="2" t="inlineStr">
         <is>
           <t>Ekscytacja</t>
         </is>
       </c>
-      <c r="F37" s="2" t="n">
+      <c r="G37" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="G37" s="2" t="inlineStr">
+      <c r="H37" s="2" t="inlineStr">
         <is>
           <t>Moment budowania pożądania</t>
         </is>
       </c>
-      <c r="H37" s="2" t="inlineStr">
+      <c r="I37" s="2" t="inlineStr">
         <is>
           <t>tak</t>
         </is>
       </c>
-      <c r="I37" s="2" t="inlineStr">
+      <c r="J37" s="2" t="inlineStr">
         <is>
           <t>Sprzedaż dealera</t>
         </is>
       </c>
-      <c r="J37" s="2" t="inlineStr">
+      <c r="K37" s="2" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="K37" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
       <c r="L37" s="2" t="inlineStr">
         <is>
-          <t>salon</t>
+          <t>DEMO</t>
         </is>
       </c>
       <c r="M37" s="2" t="n">
@@ -2898,55 +2898,55 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
+          <t>salon</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
           <t>dea-07</t>
         </is>
       </c>
-      <c r="C38" s="2" t="inlineStr">
+      <c r="D38" s="2" t="inlineStr">
         <is>
           <t>Jazda próbna</t>
         </is>
       </c>
-      <c r="D38" s="2" t="inlineStr">
+      <c r="E38" s="2" t="inlineStr">
         <is>
           <t>Zakup</t>
         </is>
       </c>
-      <c r="E38" s="2" t="inlineStr">
+      <c r="F38" s="2" t="inlineStr">
         <is>
           <t>Ekscytacja</t>
         </is>
       </c>
-      <c r="F38" s="2" t="n">
+      <c r="G38" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="G38" s="2" t="inlineStr">
+      <c r="H38" s="2" t="inlineStr">
         <is>
           <t>Pierwszy realny kontakt z autem</t>
         </is>
       </c>
-      <c r="H38" s="2" t="inlineStr">
+      <c r="I38" s="2" t="inlineStr">
         <is>
           <t>częściowo</t>
         </is>
       </c>
-      <c r="I38" s="2" t="inlineStr">
+      <c r="J38" s="2" t="inlineStr">
         <is>
           <t>Sprzedaż dealera</t>
         </is>
       </c>
-      <c r="J38" s="2" t="inlineStr">
+      <c r="K38" s="2" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="K38" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
       <c r="L38" s="2" t="inlineStr">
         <is>
-          <t>salon</t>
+          <t>DEMO</t>
         </is>
       </c>
       <c r="M38" s="2" t="n">
@@ -2962,55 +2962,55 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
+          <t>salon</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
           <t>dea-08</t>
         </is>
       </c>
-      <c r="C39" s="2" t="inlineStr">
+      <c r="D39" s="2" t="inlineStr">
         <is>
           <t>Oferta i wycena</t>
         </is>
       </c>
-      <c r="D39" s="2" t="inlineStr">
+      <c r="E39" s="2" t="inlineStr">
         <is>
           <t>Zakup</t>
         </is>
       </c>
-      <c r="E39" s="2" t="inlineStr">
+      <c r="F39" s="2" t="inlineStr">
         <is>
           <t>Napięcie</t>
         </is>
       </c>
-      <c r="F39" s="2" t="n">
+      <c r="G39" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="G39" s="2" t="inlineStr">
+      <c r="H39" s="2" t="inlineStr">
         <is>
           <t>Niejasne ceny budzą nieufność</t>
         </is>
       </c>
-      <c r="H39" s="2" t="inlineStr">
+      <c r="I39" s="2" t="inlineStr">
         <is>
           <t>nie</t>
         </is>
       </c>
-      <c r="I39" s="2" t="inlineStr">
+      <c r="J39" s="2" t="inlineStr">
         <is>
           <t>Sprzedaż dealera</t>
         </is>
       </c>
-      <c r="J39" s="2" t="inlineStr">
+      <c r="K39" s="2" t="inlineStr">
         <is>
           <t>niezaopiekowany</t>
         </is>
       </c>
-      <c r="K39" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
       <c r="L39" s="2" t="inlineStr">
         <is>
-          <t>salon</t>
+          <t>DEMO</t>
         </is>
       </c>
       <c r="M39" s="2" t="n">
@@ -3026,55 +3026,55 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
+          <t>salon</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
           <t>dea-09</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr">
+      <c r="D40" s="2" t="inlineStr">
         <is>
           <t>Negocjacje</t>
         </is>
       </c>
-      <c r="D40" s="2" t="inlineStr">
+      <c r="E40" s="2" t="inlineStr">
         <is>
           <t>Zakup</t>
         </is>
       </c>
-      <c r="E40" s="2" t="inlineStr">
+      <c r="F40" s="2" t="inlineStr">
         <is>
           <t>Napięcie</t>
         </is>
       </c>
-      <c r="F40" s="2" t="n">
+      <c r="G40" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="G40" s="2" t="inlineStr">
+      <c r="H40" s="2" t="inlineStr">
         <is>
           <t>Presja obniża komfort</t>
         </is>
       </c>
-      <c r="H40" s="2" t="inlineStr">
+      <c r="I40" s="2" t="inlineStr">
         <is>
           <t>nie</t>
         </is>
       </c>
-      <c r="I40" s="2" t="inlineStr">
+      <c r="J40" s="2" t="inlineStr">
         <is>
           <t>Sprzedaż dealera</t>
         </is>
       </c>
-      <c r="J40" s="2" t="inlineStr">
+      <c r="K40" s="2" t="inlineStr">
         <is>
           <t>niezaopiekowany</t>
         </is>
       </c>
-      <c r="K40" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
       <c r="L40" s="2" t="inlineStr">
         <is>
-          <t>salon</t>
+          <t>DEMO</t>
         </is>
       </c>
       <c r="M40" s="2" t="n">
@@ -3090,55 +3090,55 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
+          <t>salon</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
           <t>dea-10</t>
         </is>
       </c>
-      <c r="C41" s="2" t="inlineStr">
+      <c r="D41" s="2" t="inlineStr">
         <is>
           <t>Wycena auta w rozliczeniu</t>
         </is>
       </c>
-      <c r="D41" s="2" t="inlineStr">
+      <c r="E41" s="2" t="inlineStr">
         <is>
           <t>Zakup</t>
         </is>
       </c>
-      <c r="E41" s="2" t="inlineStr">
+      <c r="F41" s="2" t="inlineStr">
         <is>
           <t>Niepewność</t>
         </is>
       </c>
-      <c r="F41" s="2" t="n">
+      <c r="G41" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="G41" s="2" t="inlineStr">
+      <c r="H41" s="2" t="inlineStr">
         <is>
           <t>Różnica z oczekiwaniami frustruje</t>
         </is>
       </c>
-      <c r="H41" s="2" t="inlineStr">
+      <c r="I41" s="2" t="inlineStr">
         <is>
           <t>częściowo</t>
         </is>
       </c>
-      <c r="I41" s="2" t="inlineStr">
+      <c r="J41" s="2" t="inlineStr">
         <is>
           <t>Sprzedaż dealera</t>
         </is>
       </c>
-      <c r="J41" s="2" t="inlineStr">
+      <c r="K41" s="2" t="inlineStr">
         <is>
           <t>do_poprawy</t>
         </is>
       </c>
-      <c r="K41" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
       <c r="L41" s="2" t="inlineStr">
         <is>
-          <t>salon</t>
+          <t>DEMO</t>
         </is>
       </c>
       <c r="M41" s="2" t="n">
@@ -3154,55 +3154,55 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
+          <t>dealer</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
           <t>dea-11</t>
         </is>
       </c>
-      <c r="C42" s="2" t="inlineStr">
+      <c r="D42" s="2" t="inlineStr">
         <is>
           <t>Finansowanie u dealera</t>
         </is>
       </c>
-      <c r="D42" s="2" t="inlineStr">
+      <c r="E42" s="2" t="inlineStr">
         <is>
           <t>Finansowanie</t>
         </is>
       </c>
-      <c r="E42" s="2" t="inlineStr">
+      <c r="F42" s="2" t="inlineStr">
         <is>
           <t>Niepewność</t>
         </is>
       </c>
-      <c r="F42" s="2" t="n">
+      <c r="G42" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G42" s="2" t="inlineStr">
+      <c r="H42" s="2" t="inlineStr">
         <is>
           <t>Rozmowa o kosztach budzi napięcie</t>
         </is>
       </c>
-      <c r="H42" s="2" t="inlineStr">
+      <c r="I42" s="2" t="inlineStr">
         <is>
           <t>tak</t>
         </is>
       </c>
-      <c r="I42" s="2" t="inlineStr">
+      <c r="J42" s="2" t="inlineStr">
         <is>
           <t>Finanse dealera</t>
         </is>
       </c>
-      <c r="J42" s="2" t="inlineStr">
+      <c r="K42" s="2" t="inlineStr">
         <is>
           <t>do_poprawy</t>
         </is>
       </c>
-      <c r="K42" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
       <c r="L42" s="2" t="inlineStr">
         <is>
-          <t>dealer</t>
+          <t>DEMO</t>
         </is>
       </c>
       <c r="M42" s="2" t="n">
@@ -3218,55 +3218,55 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
+          <t>dealer</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
           <t>dea-12</t>
         </is>
       </c>
-      <c r="C43" s="2" t="inlineStr">
+      <c r="D43" s="2" t="inlineStr">
         <is>
           <t>Umowa i formalności</t>
         </is>
       </c>
-      <c r="D43" s="2" t="inlineStr">
+      <c r="E43" s="2" t="inlineStr">
         <is>
           <t>Zakup</t>
         </is>
       </c>
-      <c r="E43" s="2" t="inlineStr">
+      <c r="F43" s="2" t="inlineStr">
         <is>
           <t>Znużenie</t>
         </is>
       </c>
-      <c r="F43" s="2" t="n">
+      <c r="G43" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="G43" s="2" t="inlineStr">
+      <c r="H43" s="2" t="inlineStr">
         <is>
           <t>Papierologia osłabia emocje</t>
         </is>
       </c>
-      <c r="H43" s="2" t="inlineStr">
+      <c r="I43" s="2" t="inlineStr">
         <is>
           <t>nie</t>
         </is>
       </c>
-      <c r="I43" s="2" t="inlineStr">
+      <c r="J43" s="2" t="inlineStr">
         <is>
           <t>Sprzedaż dealera</t>
         </is>
       </c>
-      <c r="J43" s="2" t="inlineStr">
+      <c r="K43" s="2" t="inlineStr">
         <is>
           <t>niezaopiekowany</t>
         </is>
       </c>
-      <c r="K43" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
       <c r="L43" s="2" t="inlineStr">
         <is>
-          <t>dealer</t>
+          <t>DEMO</t>
         </is>
       </c>
       <c r="M43" s="2" t="n">
@@ -3282,55 +3282,55 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
+          <t>salon</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
           <t>dea-13</t>
         </is>
       </c>
-      <c r="C44" s="2" t="inlineStr">
+      <c r="D44" s="2" t="inlineStr">
         <is>
           <t>Przygotowanie auta do wydania</t>
         </is>
       </c>
-      <c r="D44" s="2" t="inlineStr">
+      <c r="E44" s="2" t="inlineStr">
         <is>
           <t>Dostawa</t>
         </is>
       </c>
-      <c r="E44" s="2" t="inlineStr">
+      <c r="F44" s="2" t="inlineStr">
         <is>
           <t>Oczekiwanie</t>
         </is>
       </c>
-      <c r="F44" s="2" t="n">
+      <c r="G44" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G44" s="2" t="inlineStr">
+      <c r="H44" s="2" t="inlineStr">
         <is>
           <t>Budzi radosne oczekiwanie</t>
         </is>
       </c>
-      <c r="H44" s="2" t="inlineStr">
+      <c r="I44" s="2" t="inlineStr">
         <is>
           <t>tak</t>
         </is>
       </c>
-      <c r="I44" s="2" t="inlineStr">
+      <c r="J44" s="2" t="inlineStr">
         <is>
           <t>Dealer</t>
         </is>
       </c>
-      <c r="J44" s="2" t="inlineStr">
+      <c r="K44" s="2" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="K44" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
       <c r="L44" s="2" t="inlineStr">
         <is>
-          <t>salon</t>
+          <t>DEMO</t>
         </is>
       </c>
       <c r="M44" s="2" t="n">
@@ -3346,55 +3346,55 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
+          <t>salon</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
           <t>dea-14</t>
         </is>
       </c>
-      <c r="C45" s="2" t="inlineStr">
+      <c r="D45" s="2" t="inlineStr">
         <is>
           <t>Wydanie auta</t>
         </is>
       </c>
-      <c r="D45" s="2" t="inlineStr">
+      <c r="E45" s="2" t="inlineStr">
         <is>
           <t>Dostawa</t>
         </is>
       </c>
-      <c r="E45" s="2" t="inlineStr">
+      <c r="F45" s="2" t="inlineStr">
         <is>
           <t>Radość</t>
         </is>
       </c>
-      <c r="F45" s="2" t="n">
+      <c r="G45" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="G45" s="2" t="inlineStr">
+      <c r="H45" s="2" t="inlineStr">
         <is>
           <t>Moment ważny emocjonalnie</t>
         </is>
       </c>
-      <c r="H45" s="2" t="inlineStr">
+      <c r="I45" s="2" t="inlineStr">
         <is>
           <t>tak</t>
         </is>
       </c>
-      <c r="I45" s="2" t="inlineStr">
+      <c r="J45" s="2" t="inlineStr">
         <is>
           <t>Dealer</t>
         </is>
       </c>
-      <c r="J45" s="2" t="inlineStr">
+      <c r="K45" s="2" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="K45" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
       <c r="L45" s="2" t="inlineStr">
         <is>
-          <t>salon</t>
+          <t>DEMO</t>
         </is>
       </c>
       <c r="M45" s="2" t="n">
@@ -3410,55 +3410,55 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
+          <t>salon</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
           <t>dea-15</t>
         </is>
       </c>
-      <c r="C46" s="2" t="inlineStr">
+      <c r="D46" s="2" t="inlineStr">
         <is>
           <t>Szkolenie z obsługi auta</t>
         </is>
       </c>
-      <c r="D46" s="2" t="inlineStr">
+      <c r="E46" s="2" t="inlineStr">
         <is>
           <t>Dostawa</t>
         </is>
       </c>
-      <c r="E46" s="2" t="inlineStr">
+      <c r="F46" s="2" t="inlineStr">
         <is>
           <t>Pewność</t>
         </is>
       </c>
-      <c r="F46" s="2" t="n">
+      <c r="G46" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G46" s="2" t="inlineStr">
+      <c r="H46" s="2" t="inlineStr">
         <is>
           <t>Daje poczucie opanowania auta</t>
         </is>
       </c>
-      <c r="H46" s="2" t="inlineStr">
+      <c r="I46" s="2" t="inlineStr">
         <is>
           <t>częściowo</t>
         </is>
       </c>
-      <c r="I46" s="2" t="inlineStr">
+      <c r="J46" s="2" t="inlineStr">
         <is>
           <t>Sprzedaż dealera</t>
         </is>
       </c>
-      <c r="J46" s="2" t="inlineStr">
+      <c r="K46" s="2" t="inlineStr">
         <is>
           <t>do_poprawy</t>
         </is>
       </c>
-      <c r="K46" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
       <c r="L46" s="2" t="inlineStr">
         <is>
-          <t>salon</t>
+          <t>DEMO</t>
         </is>
       </c>
       <c r="M46" s="2" t="n">
@@ -3474,55 +3474,55 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
+          <t>dealer</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
           <t>dea-16</t>
         </is>
       </c>
-      <c r="C47" s="2" t="inlineStr">
+      <c r="D47" s="2" t="inlineStr">
         <is>
           <t>Kontakt po 7 dniach od wydania</t>
         </is>
       </c>
-      <c r="D47" s="2" t="inlineStr">
+      <c r="E47" s="2" t="inlineStr">
         <is>
           <t>Dostawa</t>
         </is>
       </c>
-      <c r="E47" s="2" t="inlineStr">
+      <c r="F47" s="2" t="inlineStr">
         <is>
           <t>Docenienie</t>
         </is>
       </c>
-      <c r="F47" s="2" t="n">
+      <c r="G47" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G47" s="2" t="inlineStr">
+      <c r="H47" s="2" t="inlineStr">
         <is>
           <t>Pokazuje troskę o klienta</t>
         </is>
       </c>
-      <c r="H47" s="2" t="inlineStr">
+      <c r="I47" s="2" t="inlineStr">
         <is>
           <t>nie</t>
         </is>
       </c>
-      <c r="I47" s="2" t="inlineStr">
+      <c r="J47" s="2" t="inlineStr">
         <is>
           <t>Sprzedaż dealera</t>
         </is>
       </c>
-      <c r="J47" s="2" t="inlineStr">
+      <c r="K47" s="2" t="inlineStr">
         <is>
           <t>niezaopiekowany</t>
         </is>
       </c>
-      <c r="K47" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
       <c r="L47" s="2" t="inlineStr">
         <is>
-          <t>dealer</t>
+          <t>DEMO</t>
         </is>
       </c>
       <c r="M47" s="2" t="n">
@@ -3538,55 +3538,55 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
+          <t>serwis</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
           <t>dea-17</t>
         </is>
       </c>
-      <c r="C48" s="2" t="inlineStr">
+      <c r="D48" s="2" t="inlineStr">
         <is>
           <t>Rezerwacja serwisu</t>
         </is>
       </c>
-      <c r="D48" s="2" t="inlineStr">
+      <c r="E48" s="2" t="inlineStr">
         <is>
           <t>Serwis</t>
         </is>
       </c>
-      <c r="E48" s="2" t="inlineStr">
+      <c r="F48" s="2" t="inlineStr">
         <is>
           <t>Wygoda</t>
         </is>
       </c>
-      <c r="F48" s="2" t="n">
+      <c r="G48" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G48" s="2" t="inlineStr">
+      <c r="H48" s="2" t="inlineStr">
         <is>
           <t>Łatwa rezerwacja zmniejsza opór</t>
         </is>
       </c>
-      <c r="H48" s="2" t="inlineStr">
+      <c r="I48" s="2" t="inlineStr">
         <is>
           <t>częściowo</t>
         </is>
       </c>
-      <c r="I48" s="2" t="inlineStr">
+      <c r="J48" s="2" t="inlineStr">
         <is>
           <t>Serwis dealera</t>
         </is>
       </c>
-      <c r="J48" s="2" t="inlineStr">
+      <c r="K48" s="2" t="inlineStr">
         <is>
           <t>do_poprawy</t>
         </is>
       </c>
-      <c r="K48" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
       <c r="L48" s="2" t="inlineStr">
         <is>
-          <t>serwis</t>
+          <t>DEMO</t>
         </is>
       </c>
       <c r="M48" s="2" t="n">
@@ -3602,55 +3602,55 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
+          <t>serwis</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
           <t>dea-18</t>
         </is>
       </c>
-      <c r="C49" s="2" t="inlineStr">
+      <c r="D49" s="2" t="inlineStr">
         <is>
           <t>Przyjęcie do serwisu</t>
         </is>
       </c>
-      <c r="D49" s="2" t="inlineStr">
+      <c r="E49" s="2" t="inlineStr">
         <is>
           <t>Serwis</t>
         </is>
       </c>
-      <c r="E49" s="2" t="inlineStr">
+      <c r="F49" s="2" t="inlineStr">
         <is>
           <t>Niepewność</t>
         </is>
       </c>
-      <c r="F49" s="2" t="n">
+      <c r="G49" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G49" s="2" t="inlineStr">
+      <c r="H49" s="2" t="inlineStr">
         <is>
           <t>Klient nie wie co się stanie z autem</t>
         </is>
       </c>
-      <c r="H49" s="2" t="inlineStr">
+      <c r="I49" s="2" t="inlineStr">
         <is>
           <t>częściowo</t>
         </is>
       </c>
-      <c r="I49" s="2" t="inlineStr">
+      <c r="J49" s="2" t="inlineStr">
         <is>
           <t>Serwis dealera</t>
         </is>
       </c>
-      <c r="J49" s="2" t="inlineStr">
+      <c r="K49" s="2" t="inlineStr">
         <is>
           <t>do_poprawy</t>
         </is>
       </c>
-      <c r="K49" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
       <c r="L49" s="2" t="inlineStr">
         <is>
-          <t>serwis</t>
+          <t>DEMO</t>
         </is>
       </c>
       <c r="M49" s="2" t="n">
@@ -3666,55 +3666,55 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
+          <t>serwis</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
           <t>dea-19</t>
         </is>
       </c>
-      <c r="C50" s="2" t="inlineStr">
+      <c r="D50" s="2" t="inlineStr">
         <is>
           <t>Kosztorys napraw</t>
         </is>
       </c>
-      <c r="D50" s="2" t="inlineStr">
+      <c r="E50" s="2" t="inlineStr">
         <is>
           <t>Serwis</t>
         </is>
       </c>
-      <c r="E50" s="2" t="inlineStr">
+      <c r="F50" s="2" t="inlineStr">
         <is>
           <t>Niepokój</t>
         </is>
       </c>
-      <c r="F50" s="2" t="n">
+      <c r="G50" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="G50" s="2" t="inlineStr">
+      <c r="H50" s="2" t="inlineStr">
         <is>
           <t>Wysoka cena budzi obawy</t>
         </is>
       </c>
-      <c r="H50" s="2" t="inlineStr">
+      <c r="I50" s="2" t="inlineStr">
         <is>
           <t>tak</t>
         </is>
       </c>
-      <c r="I50" s="2" t="inlineStr">
+      <c r="J50" s="2" t="inlineStr">
         <is>
           <t>Serwis dealera</t>
         </is>
       </c>
-      <c r="J50" s="2" t="inlineStr">
+      <c r="K50" s="2" t="inlineStr">
         <is>
           <t>do_poprawy</t>
         </is>
       </c>
-      <c r="K50" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
       <c r="L50" s="2" t="inlineStr">
         <is>
-          <t>serwis</t>
+          <t>DEMO</t>
         </is>
       </c>
       <c r="M50" s="2" t="n">
@@ -3730,55 +3730,55 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
+          <t>serwis</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
           <t>dea-20</t>
         </is>
       </c>
-      <c r="C51" s="2" t="inlineStr">
+      <c r="D51" s="2" t="inlineStr">
         <is>
           <t>Prace dodatkowe</t>
         </is>
       </c>
-      <c r="D51" s="2" t="inlineStr">
+      <c r="E51" s="2" t="inlineStr">
         <is>
           <t>Serwis</t>
         </is>
       </c>
-      <c r="E51" s="2" t="inlineStr">
+      <c r="F51" s="2" t="inlineStr">
         <is>
           <t>Złość</t>
         </is>
       </c>
-      <c r="F51" s="2" t="n">
+      <c r="G51" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="G51" s="2" t="inlineStr">
+      <c r="H51" s="2" t="inlineStr">
         <is>
           <t>Niespodzianka kosztowa mocno obniża zaufanie</t>
         </is>
       </c>
-      <c r="H51" s="2" t="inlineStr">
+      <c r="I51" s="2" t="inlineStr">
         <is>
           <t>tak</t>
         </is>
       </c>
-      <c r="I51" s="2" t="inlineStr">
+      <c r="J51" s="2" t="inlineStr">
         <is>
           <t>Serwis dealera</t>
         </is>
       </c>
-      <c r="J51" s="2" t="inlineStr">
+      <c r="K51" s="2" t="inlineStr">
         <is>
           <t>niezaopiekowany</t>
         </is>
       </c>
-      <c r="K51" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
       <c r="L51" s="2" t="inlineStr">
         <is>
-          <t>serwis</t>
+          <t>DEMO</t>
         </is>
       </c>
       <c r="M51" s="2" t="n">
@@ -3794,55 +3794,55 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
+          <t>serwis</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
           <t>dea-21</t>
         </is>
       </c>
-      <c r="C52" s="2" t="inlineStr">
+      <c r="D52" s="2" t="inlineStr">
         <is>
           <t>Auto zastępcze</t>
         </is>
       </c>
-      <c r="D52" s="2" t="inlineStr">
+      <c r="E52" s="2" t="inlineStr">
         <is>
           <t>Serwis</t>
         </is>
       </c>
-      <c r="E52" s="2" t="inlineStr">
+      <c r="F52" s="2" t="inlineStr">
         <is>
           <t>Wdzięczność</t>
         </is>
       </c>
-      <c r="F52" s="2" t="n">
+      <c r="G52" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G52" s="2" t="inlineStr">
+      <c r="H52" s="2" t="inlineStr">
         <is>
           <t>Zmniejsza uciążliwość wizyty</t>
         </is>
       </c>
-      <c r="H52" s="2" t="inlineStr">
+      <c r="I52" s="2" t="inlineStr">
         <is>
           <t>tak</t>
         </is>
       </c>
-      <c r="I52" s="2" t="inlineStr">
+      <c r="J52" s="2" t="inlineStr">
         <is>
           <t>Serwis dealera</t>
         </is>
       </c>
-      <c r="J52" s="2" t="inlineStr">
+      <c r="K52" s="2" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="K52" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
       <c r="L52" s="2" t="inlineStr">
         <is>
-          <t>serwis</t>
+          <t>DEMO</t>
         </is>
       </c>
       <c r="M52" s="2" t="n">
@@ -3858,55 +3858,55 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
+          <t>serwis</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
           <t>dea-22</t>
         </is>
       </c>
-      <c r="C53" s="2" t="inlineStr">
+      <c r="D53" s="2" t="inlineStr">
         <is>
           <t>Poczekalnia</t>
         </is>
       </c>
-      <c r="D53" s="2" t="inlineStr">
+      <c r="E53" s="2" t="inlineStr">
         <is>
           <t>Serwis</t>
         </is>
       </c>
-      <c r="E53" s="2" t="inlineStr">
+      <c r="F53" s="2" t="inlineStr">
         <is>
           <t>Znużenie</t>
         </is>
       </c>
-      <c r="F53" s="2" t="n">
+      <c r="G53" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G53" s="2" t="inlineStr">
+      <c r="H53" s="2" t="inlineStr">
         <is>
           <t>Komfort wpływa na nastrój</t>
         </is>
       </c>
-      <c r="H53" s="2" t="inlineStr">
+      <c r="I53" s="2" t="inlineStr">
         <is>
           <t>nie</t>
         </is>
       </c>
-      <c r="I53" s="2" t="inlineStr">
+      <c r="J53" s="2" t="inlineStr">
         <is>
           <t>Serwis dealera</t>
         </is>
       </c>
-      <c r="J53" s="2" t="inlineStr">
+      <c r="K53" s="2" t="inlineStr">
         <is>
           <t>do_poprawy</t>
         </is>
       </c>
-      <c r="K53" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
       <c r="L53" s="2" t="inlineStr">
         <is>
-          <t>serwis</t>
+          <t>DEMO</t>
         </is>
       </c>
       <c r="M53" s="2" t="n">
@@ -3922,55 +3922,55 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
+          <t>serwis</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
           <t>dea-23</t>
         </is>
       </c>
-      <c r="C54" s="2" t="inlineStr">
+      <c r="D54" s="2" t="inlineStr">
         <is>
           <t>Informowanie o postępie prac</t>
         </is>
       </c>
-      <c r="D54" s="2" t="inlineStr">
+      <c r="E54" s="2" t="inlineStr">
         <is>
           <t>Serwis</t>
         </is>
       </c>
-      <c r="E54" s="2" t="inlineStr">
+      <c r="F54" s="2" t="inlineStr">
         <is>
           <t>Niecierpliwość</t>
         </is>
       </c>
-      <c r="F54" s="2" t="n">
+      <c r="G54" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="G54" s="2" t="inlineStr">
+      <c r="H54" s="2" t="inlineStr">
         <is>
           <t>Brak informacji wydłuża oczekiwanie</t>
         </is>
       </c>
-      <c r="H54" s="2" t="inlineStr">
+      <c r="I54" s="2" t="inlineStr">
         <is>
           <t>nie</t>
         </is>
       </c>
-      <c r="I54" s="2" t="inlineStr">
+      <c r="J54" s="2" t="inlineStr">
         <is>
           <t>Serwis dealera</t>
         </is>
       </c>
-      <c r="J54" s="2" t="inlineStr">
+      <c r="K54" s="2" t="inlineStr">
         <is>
           <t>niezaopiekowany</t>
         </is>
       </c>
-      <c r="K54" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
       <c r="L54" s="2" t="inlineStr">
         <is>
-          <t>serwis</t>
+          <t>DEMO</t>
         </is>
       </c>
       <c r="M54" s="2" t="n">
@@ -3986,45 +3986,45 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
+          <t>serwis</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
           <t>dea-24</t>
         </is>
       </c>
-      <c r="C55" s="2" t="inlineStr">
+      <c r="D55" s="2" t="inlineStr">
         <is>
           <t>Odbiór po serwisie</t>
         </is>
       </c>
-      <c r="D55" s="2" t="inlineStr">
+      <c r="E55" s="2" t="inlineStr">
         <is>
           <t>Serwis</t>
         </is>
       </c>
-      <c r="E55" s="2" t="inlineStr"/>
       <c r="F55" s="2" t="inlineStr"/>
       <c r="G55" s="2" t="inlineStr"/>
-      <c r="H55" s="2" t="inlineStr">
+      <c r="H55" s="2" t="inlineStr"/>
+      <c r="I55" s="2" t="inlineStr">
         <is>
           <t>nie</t>
         </is>
       </c>
-      <c r="I55" s="2" t="inlineStr">
+      <c r="J55" s="2" t="inlineStr">
         <is>
           <t>Serwis dealera</t>
         </is>
       </c>
-      <c r="J55" s="2" t="inlineStr">
+      <c r="K55" s="2" t="inlineStr">
         <is>
           <t>brak_oceny</t>
         </is>
       </c>
-      <c r="K55" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
       <c r="L55" s="2" t="inlineStr">
         <is>
-          <t>serwis</t>
+          <t>DEMO</t>
         </is>
       </c>
       <c r="M55" s="2" t="inlineStr"/>
@@ -4038,55 +4038,55 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
+          <t>serwis</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
           <t>dea-25</t>
         </is>
       </c>
-      <c r="C56" s="2" t="inlineStr">
+      <c r="D56" s="2" t="inlineStr">
         <is>
           <t>Rozliczenie i faktura</t>
         </is>
       </c>
-      <c r="D56" s="2" t="inlineStr">
+      <c r="E56" s="2" t="inlineStr">
         <is>
           <t>Serwis</t>
         </is>
       </c>
-      <c r="E56" s="2" t="inlineStr">
+      <c r="F56" s="2" t="inlineStr">
         <is>
           <t>Obojętność</t>
         </is>
       </c>
-      <c r="F56" s="2" t="n">
+      <c r="G56" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G56" s="2" t="inlineStr">
+      <c r="H56" s="2" t="inlineStr">
         <is>
           <t>Neutralne gdy zgodne z ofertą</t>
         </is>
       </c>
-      <c r="H56" s="2" t="inlineStr">
+      <c r="I56" s="2" t="inlineStr">
         <is>
           <t>tak</t>
         </is>
       </c>
-      <c r="I56" s="2" t="inlineStr">
+      <c r="J56" s="2" t="inlineStr">
         <is>
           <t>Serwis dealera</t>
         </is>
       </c>
-      <c r="J56" s="2" t="inlineStr">
+      <c r="K56" s="2" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="K56" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
       <c r="L56" s="2" t="inlineStr">
         <is>
-          <t>serwis</t>
+          <t>DEMO</t>
         </is>
       </c>
       <c r="M56" s="2" t="n">
@@ -4102,55 +4102,55 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
+          <t>serwis</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
           <t>dea-26</t>
         </is>
       </c>
-      <c r="C57" s="2" t="inlineStr">
+      <c r="D57" s="2" t="inlineStr">
         <is>
           <t>Kontakt po serwisie</t>
         </is>
       </c>
-      <c r="D57" s="2" t="inlineStr">
+      <c r="E57" s="2" t="inlineStr">
         <is>
           <t>Serwis</t>
         </is>
       </c>
-      <c r="E57" s="2" t="inlineStr">
+      <c r="F57" s="2" t="inlineStr">
         <is>
           <t>Docenienie</t>
         </is>
       </c>
-      <c r="F57" s="2" t="n">
+      <c r="G57" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G57" s="2" t="inlineStr">
+      <c r="H57" s="2" t="inlineStr">
         <is>
           <t>Pokazuje troskę o klienta</t>
         </is>
       </c>
-      <c r="H57" s="2" t="inlineStr">
+      <c r="I57" s="2" t="inlineStr">
         <is>
           <t>nie</t>
         </is>
       </c>
-      <c r="I57" s="2" t="inlineStr">
+      <c r="J57" s="2" t="inlineStr">
         <is>
           <t>Serwis dealera</t>
         </is>
       </c>
-      <c r="J57" s="2" t="inlineStr">
+      <c r="K57" s="2" t="inlineStr">
         <is>
           <t>niezaopiekowany</t>
         </is>
       </c>
-      <c r="K57" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
       <c r="L57" s="2" t="inlineStr">
         <is>
-          <t>serwis</t>
+          <t>DEMO</t>
         </is>
       </c>
       <c r="M57" s="2" t="n">
@@ -4166,55 +4166,55 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
+          <t>serwis</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
           <t>dea-27</t>
         </is>
       </c>
-      <c r="C58" s="2" t="inlineStr">
+      <c r="D58" s="2" t="inlineStr">
         <is>
           <t>Naprawa gwarancyjna</t>
         </is>
       </c>
-      <c r="D58" s="2" t="inlineStr">
+      <c r="E58" s="2" t="inlineStr">
         <is>
           <t>Gwarancja</t>
         </is>
       </c>
-      <c r="E58" s="2" t="inlineStr">
+      <c r="F58" s="2" t="inlineStr">
         <is>
           <t>Napięcie</t>
         </is>
       </c>
-      <c r="F58" s="2" t="n">
+      <c r="G58" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="G58" s="2" t="inlineStr">
+      <c r="H58" s="2" t="inlineStr">
         <is>
           <t>Spór o gwarancję obniża zaufanie</t>
         </is>
       </c>
-      <c r="H58" s="2" t="inlineStr">
+      <c r="I58" s="2" t="inlineStr">
         <is>
           <t>tak</t>
         </is>
       </c>
-      <c r="I58" s="2" t="inlineStr">
+      <c r="J58" s="2" t="inlineStr">
         <is>
           <t>Serwis dealera</t>
         </is>
       </c>
-      <c r="J58" s="2" t="inlineStr">
+      <c r="K58" s="2" t="inlineStr">
         <is>
           <t>do_poprawy</t>
         </is>
       </c>
-      <c r="K58" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
       <c r="L58" s="2" t="inlineStr">
         <is>
-          <t>serwis</t>
+          <t>DEMO</t>
         </is>
       </c>
       <c r="M58" s="2" t="n">
@@ -4230,55 +4230,55 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
+          <t>serwis</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
           <t>dea-28</t>
         </is>
       </c>
-      <c r="C59" s="2" t="inlineStr">
+      <c r="D59" s="2" t="inlineStr">
         <is>
           <t>Naprawa blacharska po wypadku</t>
         </is>
       </c>
-      <c r="D59" s="2" t="inlineStr">
+      <c r="E59" s="2" t="inlineStr">
         <is>
           <t>Serwis</t>
         </is>
       </c>
-      <c r="E59" s="2" t="inlineStr">
+      <c r="F59" s="2" t="inlineStr">
         <is>
           <t>Stres</t>
         </is>
       </c>
-      <c r="F59" s="2" t="n">
+      <c r="G59" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="G59" s="2" t="inlineStr">
+      <c r="H59" s="2" t="inlineStr">
         <is>
           <t>Trudna sytuacja życiowa klienta</t>
         </is>
       </c>
-      <c r="H59" s="2" t="inlineStr">
+      <c r="I59" s="2" t="inlineStr">
         <is>
           <t>częściowo</t>
         </is>
       </c>
-      <c r="I59" s="2" t="inlineStr">
+      <c r="J59" s="2" t="inlineStr">
         <is>
           <t>Serwis dealera</t>
         </is>
       </c>
-      <c r="J59" s="2" t="inlineStr">
+      <c r="K59" s="2" t="inlineStr">
         <is>
           <t>do_poprawy</t>
         </is>
       </c>
-      <c r="K59" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
       <c r="L59" s="2" t="inlineStr">
         <is>
-          <t>serwis</t>
+          <t>DEMO</t>
         </is>
       </c>
       <c r="M59" s="2" t="n">
@@ -4294,55 +4294,55 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
+          <t>dealer</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
           <t>dea-29</t>
         </is>
       </c>
-      <c r="C60" s="2" t="inlineStr">
+      <c r="D60" s="2" t="inlineStr">
         <is>
           <t>Sprzedaż samochodów używanych</t>
         </is>
       </c>
-      <c r="D60" s="2" t="inlineStr">
+      <c r="E60" s="2" t="inlineStr">
         <is>
           <t>Auta używane</t>
         </is>
       </c>
-      <c r="E60" s="2" t="inlineStr">
+      <c r="F60" s="2" t="inlineStr">
         <is>
           <t>Nieufność</t>
         </is>
       </c>
-      <c r="F60" s="2" t="n">
+      <c r="G60" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="G60" s="2" t="inlineStr">
+      <c r="H60" s="2" t="inlineStr">
         <is>
           <t>Niska pewność co do stanu auta</t>
         </is>
       </c>
-      <c r="H60" s="2" t="inlineStr">
+      <c r="I60" s="2" t="inlineStr">
         <is>
           <t>nie</t>
         </is>
       </c>
-      <c r="I60" s="2" t="inlineStr">
+      <c r="J60" s="2" t="inlineStr">
         <is>
           <t>Sprzedaż dealera</t>
         </is>
       </c>
-      <c r="J60" s="2" t="inlineStr">
+      <c r="K60" s="2" t="inlineStr">
         <is>
           <t>niezaopiekowany</t>
         </is>
       </c>
-      <c r="K60" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
       <c r="L60" s="2" t="inlineStr">
         <is>
-          <t>dealer</t>
+          <t>DEMO</t>
         </is>
       </c>
       <c r="M60" s="2" t="n">
@@ -4358,55 +4358,55 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
+          <t>dealer</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
           <t>dea-30</t>
         </is>
       </c>
-      <c r="C61" s="2" t="inlineStr">
+      <c r="D61" s="2" t="inlineStr">
         <is>
           <t>Kontakt przed końcem umowy</t>
         </is>
       </c>
-      <c r="D61" s="2" t="inlineStr">
+      <c r="E61" s="2" t="inlineStr">
         <is>
           <t>Lojalność</t>
         </is>
       </c>
-      <c r="E61" s="2" t="inlineStr">
+      <c r="F61" s="2" t="inlineStr">
         <is>
           <t>Zainteresowanie</t>
         </is>
       </c>
-      <c r="F61" s="2" t="n">
+      <c r="G61" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G61" s="2" t="inlineStr">
+      <c r="H61" s="2" t="inlineStr">
         <is>
           <t>Szansa na kolejną sprzedaż</t>
         </is>
       </c>
-      <c r="H61" s="2" t="inlineStr">
+      <c r="I61" s="2" t="inlineStr">
         <is>
           <t>nie</t>
         </is>
       </c>
-      <c r="I61" s="2" t="inlineStr">
+      <c r="J61" s="2" t="inlineStr">
         <is>
           <t>Sprzedaż dealera</t>
         </is>
       </c>
-      <c r="J61" s="2" t="inlineStr">
+      <c r="K61" s="2" t="inlineStr">
         <is>
           <t>niezaopiekowany</t>
         </is>
       </c>
-      <c r="K61" s="2" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
       <c r="L61" s="2" t="inlineStr">
         <is>
-          <t>dealer</t>
+          <t>DEMO</t>
         </is>
       </c>
       <c r="M61" s="2" t="n">
@@ -4420,19 +4420,19 @@
     <dataValidation sqref="A2:A1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Macierz" error="Wybierz wartość z listy (słownik)." type="list">
       <formula1>=slowniki!$B$2:$B$3</formula1>
     </dataValidation>
-    <dataValidation sqref="L2:L1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Podtyp" error="Wybierz wartość z listy (słownik) albo zostaw puste." type="list">
+    <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Podtyp" error="Wybierz wartość z listy (słownik) albo zostaw puste." type="list">
       <formula1>=slowniki!$B$4:$B$6</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Ocena CX" error="Wybierz wartość z listy (słownik)." type="list">
+    <dataValidation sqref="K2:K1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Ocena CX" error="Wybierz wartość z listy (słownik)." type="list">
       <formula1>=slowniki!$B$7:$B$10</formula1>
     </dataValidation>
-    <dataValidation sqref="H2:H1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Monitoring" error="Wybierz wartość z listy (słownik)." type="list">
+    <dataValidation sqref="I2:I1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Monitoring" error="Wybierz wartość z listy (słownik)." type="list">
       <formula1>=slowniki!$B$11:$B$13</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Proces" error="Wybierz proces z zakładki procesy." type="list">
+    <dataValidation sqref="E2:E1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Proces" error="Wybierz proces z zakładki procesy." type="list">
       <formula1>=procesy!$B$2:$B$1000</formula1>
     </dataValidation>
-    <dataValidation sqref="F2:F1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Skala 1-5" error="Wpisz liczbę całkowitą od 1 do 5." type="whole" operator="between">
+    <dataValidation sqref="G2:G1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Skala 1-5" error="Wpisz liczbę całkowitą od 1 do 5." type="whole" operator="between">
       <formula1>1</formula1>
       <formula2>5</formula2>
     </dataValidation>
@@ -14186,7 +14186,7 @@
   <autoFilter ref="A1:E360"/>
   <dataValidations count="2">
     <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Punkt" error="Wybierz ID z zakładki punkty_styku." type="list">
-      <formula1>=punkty_styku!$B$2:$B$1000</formula1>
+      <formula1>=punkty_styku!$C$2:$C$1000</formula1>
     </dataValidation>
     <dataValidation sqref="C2:C1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Typ cechy" error="Wybierz wartość z listy (słownik)." type="list">
       <formula1>=slowniki!$B$14:$B$18</formula1>
@@ -17024,7 +17024,7 @@
   <autoFilter ref="A1:J56"/>
   <dataValidations count="6">
     <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Punkt" error="Wybierz ID z zakładki punkty_styku." type="list">
-      <formula1>=punkty_styku!$B$2:$B$1000</formula1>
+      <formula1>=punkty_styku!$C$2:$C$1000</formula1>
     </dataValidation>
     <dataValidation sqref="C2:C1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Rodzaj akcji" error="Wybierz wartość z listy (słownik)." type="list">
       <formula1>=slowniki!$B$19:$B$20</formula1>
@@ -19669,10 +19669,10 @@
   <autoFilter ref="A1:E84"/>
   <dataValidations count="3">
     <dataValidation sqref="A2:A1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Punkt" error="Wybierz ID z zakładki punkty_styku." type="list">
-      <formula1>=punkty_styku!$B$2:$B$1000</formula1>
+      <formula1>=punkty_styku!$C$2:$C$1000</formula1>
     </dataValidation>
     <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Punkt" error="Wybierz ID z zakładki punkty_styku." type="list">
-      <formula1>=punkty_styku!$B$2:$B$1000</formula1>
+      <formula1>=punkty_styku!$C$2:$C$1000</formula1>
     </dataValidation>
     <dataValidation sqref="D2:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Opcjonalny" error="Wybierz: tak albo nie (puste = nie)." type="list">
       <formula1>"tak,nie"</formula1>
@@ -20779,7 +20779,7 @@
       <formula1>=przypadki!$A$2:$A$1000</formula1>
     </dataValidation>
     <dataValidation sqref="C2:C1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Punkt" error="Wybierz ID z zakładki punkty_styku." type="list">
-      <formula1>=punkty_styku!$B$2:$B$1000</formula1>
+      <formula1>=punkty_styku!$C$2:$C$1000</formula1>
     </dataValidation>
     <dataValidation sqref="D2:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Stan" error="Wybierz wartość z listy (słownik)." type="list">
       <formula1>=slowniki!$B$21:$B$24</formula1>

</xml_diff>